<commit_message>
Sync from OneDrive: SUrsini_2026TimeTracking.xlsx [2026-04-09 15:25 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ctbuh.sharepoint.com/sites/Staff/Shared Documents/Research/Time Tracking/2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2588" documentId="8_{19902409-0CA0-44C6-BB05-58D04BF4FCB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4178A822-214D-4B5A-AE2D-AE2DCC41A4ED}"/>
+  <xr:revisionPtr revIDLastSave="2602" documentId="8_{19902409-0CA0-44C6-BB05-58D04BF4FCB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4AFD286C-10FC-46D9-BFF1-8CD6E5FC2E7C}"/>
   <bookViews>
     <workbookView xWindow="-38400" yWindow="11600" windowWidth="19000" windowHeight="12400" xr2:uid="{0C10F557-92E5-4EB6-9E48-62A8B86D346C}"/>
   </bookViews>
@@ -1132,11 +1132,11 @@
       </c>
       <c r="BR1" s="11">
         <f>SUM(BR$7:BR$1048576)</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="BS1" s="11">
         <f>SUM(BS$7:BS$1048576)</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="BT1" s="11">
         <f>SUM(BT$7:BT$1048576)</f>
@@ -2182,11 +2182,11 @@
       </c>
       <c r="BR2" s="11">
         <f>SUM(BR$7:BR$1048576)</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="BS2" s="11">
         <f>SUM(BS$7:BS$1048576)</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="BT2" s="11">
         <f>SUM(BT$7:BT$1048576)</f>
@@ -6902,7 +6902,7 @@
       </c>
       <c r="B7" s="13">
         <f>SUM(B8:B24)</f>
-        <v>92</v>
+        <v>100.25</v>
       </c>
       <c r="C7" s="8"/>
       <c r="D7" s="8"/>
@@ -7982,7 +7982,7 @@
       </c>
       <c r="B11" s="8">
         <f t="shared" si="15"/>
-        <v>21.5</v>
+        <v>23.25</v>
       </c>
       <c r="C11" s="8"/>
       <c r="D11" s="8"/>
@@ -8082,7 +8082,9 @@
       <c r="BQ11" s="12">
         <v>0.25</v>
       </c>
-      <c r="BR11" s="12"/>
+      <c r="BR11" s="12">
+        <v>1.75</v>
+      </c>
       <c r="BS11" s="12"/>
       <c r="BT11" s="12"/>
       <c r="BU11" s="12"/>
@@ -10183,7 +10185,7 @@
       </c>
       <c r="B19" s="8">
         <f t="shared" si="15"/>
-        <v>64.5</v>
+        <v>71</v>
       </c>
       <c r="C19" s="8"/>
       <c r="D19" s="8"/>
@@ -10286,8 +10288,12 @@
       <c r="BQ19" s="12">
         <v>0.25</v>
       </c>
-      <c r="BR19" s="12"/>
-      <c r="BS19" s="12"/>
+      <c r="BR19" s="12">
+        <v>1.5</v>
+      </c>
+      <c r="BS19" s="12">
+        <v>5</v>
+      </c>
       <c r="BT19" s="12"/>
       <c r="BU19" s="12"/>
       <c r="BV19" s="12"/>
@@ -13993,7 +13999,7 @@
       </c>
       <c r="B33" s="8">
         <f t="shared" si="15"/>
-        <v>13.5</v>
+        <v>14.5</v>
       </c>
       <c r="C33" s="23"/>
       <c r="D33" s="23"/>
@@ -14074,7 +14080,9 @@
       <c r="BQ33" s="21">
         <v>7</v>
       </c>
-      <c r="BR33" s="21"/>
+      <c r="BR33" s="21">
+        <v>1</v>
+      </c>
       <c r="BS33" s="21"/>
       <c r="BT33" s="21"/>
       <c r="BU33" s="21"/>
@@ -17476,7 +17484,7 @@
       </c>
       <c r="B46" s="8">
         <f t="shared" si="15"/>
-        <v>22.25</v>
+        <v>22.75</v>
       </c>
       <c r="C46" s="23"/>
       <c r="D46" s="23">
@@ -17579,7 +17587,9 @@
       <c r="BO46" s="21"/>
       <c r="BP46" s="21"/>
       <c r="BQ46" s="21"/>
-      <c r="BR46" s="21"/>
+      <c r="BR46" s="21">
+        <v>0.5</v>
+      </c>
       <c r="BS46" s="21"/>
       <c r="BT46" s="21"/>
       <c r="BU46" s="21"/>
@@ -18070,7 +18080,7 @@
       </c>
       <c r="B48" s="8">
         <f t="shared" si="15"/>
-        <v>71.75</v>
+        <v>73.75</v>
       </c>
       <c r="C48" s="23"/>
       <c r="D48" s="23">
@@ -18247,8 +18257,12 @@
       <c r="BQ48" s="21">
         <v>0.25</v>
       </c>
-      <c r="BR48" s="21"/>
-      <c r="BS48" s="21"/>
+      <c r="BR48" s="21">
+        <v>1</v>
+      </c>
+      <c r="BS48" s="21">
+        <v>1</v>
+      </c>
       <c r="BT48" s="21"/>
       <c r="BU48" s="21"/>
       <c r="BV48" s="21"/>
@@ -19525,7 +19539,7 @@
       </c>
       <c r="B53" s="8">
         <f t="shared" si="15"/>
-        <v>47</v>
+        <v>47.25</v>
       </c>
       <c r="C53" s="23"/>
       <c r="D53" s="23"/>
@@ -19642,7 +19656,9 @@
       <c r="BO53" s="21"/>
       <c r="BP53" s="21"/>
       <c r="BQ53" s="21"/>
-      <c r="BR53" s="21"/>
+      <c r="BR53" s="21">
+        <v>0.25</v>
+      </c>
       <c r="BS53" s="21"/>
       <c r="BT53" s="21"/>
       <c r="BU53" s="21"/>
@@ -23367,7 +23383,7 @@
       </c>
       <c r="B67" s="8">
         <f t="shared" si="15"/>
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="C67" s="23"/>
       <c r="D67" s="23"/>
@@ -23452,8 +23468,12 @@
         <v>0.5</v>
       </c>
       <c r="BQ67" s="21"/>
-      <c r="BR67" s="21"/>
-      <c r="BS67" s="21"/>
+      <c r="BR67" s="21">
+        <v>2</v>
+      </c>
+      <c r="BS67" s="21">
+        <v>2</v>
+      </c>
       <c r="BT67" s="21"/>
       <c r="BU67" s="21"/>
       <c r="BV67" s="21"/>
@@ -31545,26 +31565,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="be2d32d5-45e4-45f8-8cca-e731efdae529">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008A7894324D7C3949B4D325554D1FC6DA" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="43dd22c4a0a55be49439aa2cba9a6031">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="be2d32d5-45e4-45f8-8cca-e731efdae529" xmlns:ns3="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="67300191881baa0ec8105967d66c0489" ns2:_="" ns3:_="">
     <xsd:import namespace="be2d32d5-45e4-45f8-8cca-e731efdae529"/>
@@ -31805,8 +31805,28 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="be2d32d5-45e4-45f8-8cca-e731efdae529">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{035973C1-EA40-447A-BB47-72CAA2093BEE}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{99FF388B-5428-4A7E-9E36-70DDEC026763}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -31814,5 +31834,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{99FF388B-5428-4A7E-9E36-70DDEC026763}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{035973C1-EA40-447A-BB47-72CAA2093BEE}"/>
 </file>
</xml_diff>

<commit_message>
Sync from OneDrive: SUrsini_2026TimeTracking.xlsx [2026-04-13 16:00 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29930"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30002"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ctbuh.sharepoint.com/sites/Staff/Shared Documents/Research/Time Tracking/2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2602" documentId="8_{19902409-0CA0-44C6-BB05-58D04BF4FCB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4AFD286C-10FC-46D9-BFF1-8CD6E5FC2E7C}"/>
+  <xr:revisionPtr revIDLastSave="2622" documentId="8_{19902409-0CA0-44C6-BB05-58D04BF4FCB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FF5C9BFA-64CE-409D-9F51-7304D79F9B12}"/>
   <bookViews>
     <workbookView xWindow="-38400" yWindow="11600" windowWidth="19000" windowHeight="12400" xr2:uid="{0C10F557-92E5-4EB6-9E48-62A8B86D346C}"/>
   </bookViews>
@@ -1140,19 +1140,19 @@
       </c>
       <c r="BT1" s="11">
         <f>SUM(BT$7:BT$1048576)</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="BU1" s="11">
         <f>SUM(BU$7:BU$1048576)</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="BV1" s="11">
         <f>SUM(BV$7:BV$1048576)</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="BW1" s="11">
         <f>SUM(BW$7:BW$1048576)</f>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="BX1" s="11">
         <f>SUM(BX$7:BX$1048576)</f>
@@ -2190,19 +2190,19 @@
       </c>
       <c r="BT2" s="11">
         <f>SUM(BT$7:BT$1048576)</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="BU2" s="11">
         <f>SUM(BU$7:BU$1048576)</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="BV2" s="11">
         <f>SUM(BV$7:BV$1048576)</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="BW2" s="11">
         <f>SUM(BW$7:BW$1048576)</f>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="BX2" s="11">
         <f>SUM(BX$7:BX$1048576)</f>
@@ -6902,7 +6902,7 @@
       </c>
       <c r="B7" s="13">
         <f>SUM(B8:B24)</f>
-        <v>100.25</v>
+        <v>116.25</v>
       </c>
       <c r="C7" s="8"/>
       <c r="D7" s="8"/>
@@ -7982,7 +7982,7 @@
       </c>
       <c r="B11" s="8">
         <f t="shared" si="15"/>
-        <v>23.25</v>
+        <v>23.75</v>
       </c>
       <c r="C11" s="8"/>
       <c r="D11" s="8"/>
@@ -8087,8 +8087,12 @@
       </c>
       <c r="BS11" s="12"/>
       <c r="BT11" s="12"/>
-      <c r="BU11" s="12"/>
-      <c r="BV11" s="12"/>
+      <c r="BU11" s="12">
+        <v>0.25</v>
+      </c>
+      <c r="BV11" s="12">
+        <v>0.25</v>
+      </c>
       <c r="BW11" s="12"/>
       <c r="BX11" s="12"/>
       <c r="BY11" s="12"/>
@@ -10185,7 +10189,7 @@
       </c>
       <c r="B19" s="8">
         <f t="shared" si="15"/>
-        <v>71</v>
+        <v>86.5</v>
       </c>
       <c r="C19" s="8"/>
       <c r="D19" s="8"/>
@@ -10294,9 +10298,15 @@
       <c r="BS19" s="12">
         <v>5</v>
       </c>
-      <c r="BT19" s="12"/>
-      <c r="BU19" s="12"/>
-      <c r="BV19" s="12"/>
+      <c r="BT19" s="12">
+        <v>4.75</v>
+      </c>
+      <c r="BU19" s="12">
+        <v>6.25</v>
+      </c>
+      <c r="BV19" s="12">
+        <v>4.5</v>
+      </c>
       <c r="BW19" s="12"/>
       <c r="BX19" s="12"/>
       <c r="BY19" s="12"/>
@@ -18080,7 +18090,7 @@
       </c>
       <c r="B48" s="8">
         <f t="shared" si="15"/>
-        <v>73.75</v>
+        <v>78.25</v>
       </c>
       <c r="C48" s="23"/>
       <c r="D48" s="23">
@@ -18263,9 +18273,15 @@
       <c r="BS48" s="21">
         <v>1</v>
       </c>
-      <c r="BT48" s="21"/>
-      <c r="BU48" s="21"/>
-      <c r="BV48" s="21"/>
+      <c r="BT48" s="21">
+        <v>1</v>
+      </c>
+      <c r="BU48" s="21">
+        <v>1</v>
+      </c>
+      <c r="BV48" s="21">
+        <v>2.5</v>
+      </c>
       <c r="BW48" s="21"/>
       <c r="BX48" s="21"/>
       <c r="BY48" s="21"/>
@@ -19539,7 +19555,7 @@
       </c>
       <c r="B53" s="8">
         <f t="shared" si="15"/>
-        <v>47.25</v>
+        <v>47.75</v>
       </c>
       <c r="C53" s="23"/>
       <c r="D53" s="23"/>
@@ -19660,9 +19676,13 @@
         <v>0.25</v>
       </c>
       <c r="BS53" s="21"/>
-      <c r="BT53" s="21"/>
+      <c r="BT53" s="21">
+        <v>0.25</v>
+      </c>
       <c r="BU53" s="21"/>
-      <c r="BV53" s="21"/>
+      <c r="BV53" s="21">
+        <v>0.25</v>
+      </c>
       <c r="BW53" s="21"/>
       <c r="BX53" s="21"/>
       <c r="BY53" s="21"/>
@@ -23383,7 +23403,7 @@
       </c>
       <c r="B67" s="8">
         <f t="shared" si="15"/>
-        <v>13</v>
+        <v>13.5</v>
       </c>
       <c r="C67" s="23"/>
       <c r="D67" s="23"/>
@@ -23474,7 +23494,9 @@
       <c r="BS67" s="21">
         <v>2</v>
       </c>
-      <c r="BT67" s="21"/>
+      <c r="BT67" s="21">
+        <v>0.5</v>
+      </c>
       <c r="BU67" s="21"/>
       <c r="BV67" s="21"/>
       <c r="BW67" s="21"/>
@@ -23673,7 +23695,7 @@
       </c>
       <c r="B68" s="8">
         <f t="shared" si="15"/>
-        <v>114.5</v>
+        <v>115.75</v>
       </c>
       <c r="C68" s="23"/>
       <c r="D68" s="23"/>
@@ -23816,10 +23838,18 @@
       <c r="BQ68" s="21"/>
       <c r="BR68" s="21"/>
       <c r="BS68" s="21"/>
-      <c r="BT68" s="21"/>
-      <c r="BU68" s="21"/>
-      <c r="BV68" s="21"/>
-      <c r="BW68" s="21"/>
+      <c r="BT68" s="21">
+        <v>0.5</v>
+      </c>
+      <c r="BU68" s="21">
+        <v>0.25</v>
+      </c>
+      <c r="BV68" s="21">
+        <v>0.25</v>
+      </c>
+      <c r="BW68" s="21">
+        <v>0.25</v>
+      </c>
       <c r="BX68" s="21"/>
       <c r="BY68" s="21"/>
       <c r="BZ68" s="21"/>
@@ -25903,7 +25933,7 @@
       </c>
       <c r="B76" s="8">
         <f t="shared" ref="B76:B78" si="16">SUM($C76:$XFD76)</f>
-        <v>14.75</v>
+        <v>16.25</v>
       </c>
       <c r="C76" s="23"/>
       <c r="D76" s="23">
@@ -26050,9 +26080,15 @@
       </c>
       <c r="BR76" s="21"/>
       <c r="BS76" s="21"/>
-      <c r="BT76" s="21"/>
-      <c r="BU76" s="21"/>
-      <c r="BV76" s="21"/>
+      <c r="BT76" s="21">
+        <v>1</v>
+      </c>
+      <c r="BU76" s="21">
+        <v>0.25</v>
+      </c>
+      <c r="BV76" s="21">
+        <v>0.25</v>
+      </c>
       <c r="BW76" s="21"/>
       <c r="BX76" s="21"/>
       <c r="BY76" s="21"/>
@@ -31565,6 +31601,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008A7894324D7C3949B4D325554D1FC6DA" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="43dd22c4a0a55be49439aa2cba9a6031">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="be2d32d5-45e4-45f8-8cca-e731efdae529" xmlns:ns3="ea83d0c8-5d24-4b4f-b406-3ee575ee00f6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="67300191881baa0ec8105967d66c0489" ns2:_="" ns3:_="">
     <xsd:import namespace="be2d32d5-45e4-45f8-8cca-e731efdae529"/>
@@ -31805,15 +31850,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -31826,11 +31862,11 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{99FF388B-5428-4A7E-9E36-70DDEC026763}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CEFE62B7-6772-44D0-ACCE-A546E807D9BB}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CEFE62B7-6772-44D0-ACCE-A546E807D9BB}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{99FF388B-5428-4A7E-9E36-70DDEC026763}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-04-21 22:42 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -17408,7 +17408,9 @@
       <c r="BU46" s="21" t="n"/>
       <c r="BV46" s="21" t="n"/>
       <c r="BW46" s="21" t="n"/>
-      <c r="BX46" s="21" t="n"/>
+      <c r="BX46" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="BY46" s="21" t="n"/>
       <c r="BZ46" s="21" t="n"/>
       <c r="CA46" s="21" t="n"/>
@@ -18092,7 +18094,9 @@
       <c r="BW48" s="21" t="n">
         <v>1.25</v>
       </c>
-      <c r="BX48" s="21" t="n"/>
+      <c r="BX48" s="21" t="n">
+        <v>1</v>
+      </c>
       <c r="BY48" s="21" t="n"/>
       <c r="BZ48" s="21" t="n"/>
       <c r="CA48" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-04-21 22:43 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -19507,7 +19507,9 @@
         <v>0.25</v>
       </c>
       <c r="BW53" s="21" t="n"/>
-      <c r="BX53" s="21" t="n"/>
+      <c r="BX53" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="BY53" s="21" t="n"/>
       <c r="BZ53" s="21" t="n"/>
       <c r="CA53" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-04-21 22:48 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -7826,7 +7826,9 @@
         <v>1.5</v>
       </c>
       <c r="BX11" s="12" t="n"/>
-      <c r="BY11" s="12" t="n"/>
+      <c r="BY11" s="12" t="n">
+        <v>0.25</v>
+      </c>
       <c r="BZ11" s="12" t="n"/>
       <c r="CA11" s="12" t="n"/>
       <c r="CB11" s="12" t="n"/>
@@ -10058,7 +10060,9 @@
         <v>5</v>
       </c>
       <c r="BX19" s="12" t="n"/>
-      <c r="BY19" s="12" t="n"/>
+      <c r="BY19" s="12" t="n">
+        <v>5.25</v>
+      </c>
       <c r="BZ19" s="12" t="n"/>
       <c r="CA19" s="12" t="n"/>
       <c r="CB19" s="12" t="n"/>
@@ -18097,7 +18101,9 @@
       <c r="BX48" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="BY48" s="21" t="n"/>
+      <c r="BY48" s="21" t="n">
+        <v>1.25</v>
+      </c>
       <c r="BZ48" s="21" t="n"/>
       <c r="CA48" s="21" t="n"/>
       <c r="CB48" s="21" t="n"/>
@@ -19510,7 +19516,9 @@
       <c r="BX53" s="21" t="n">
         <v>0.25</v>
       </c>
-      <c r="BY53" s="21" t="n"/>
+      <c r="BY53" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="BZ53" s="21" t="n"/>
       <c r="CA53" s="21" t="n"/>
       <c r="CB53" s="21" t="n"/>
@@ -23706,7 +23714,9 @@
         <v>0.25</v>
       </c>
       <c r="BX68" s="21" t="n"/>
-      <c r="BY68" s="21" t="n"/>
+      <c r="BY68" s="21" t="n">
+        <v>0.75</v>
+      </c>
       <c r="BZ68" s="21" t="n"/>
       <c r="CA68" s="21" t="n"/>
       <c r="CB68" s="21" t="n"/>
@@ -25962,7 +25972,9 @@
       </c>
       <c r="BW76" s="21" t="n"/>
       <c r="BX76" s="21" t="n"/>
-      <c r="BY76" s="21" t="n"/>
+      <c r="BY76" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="BZ76" s="21" t="n"/>
       <c r="CA76" s="21" t="n"/>
       <c r="CB76" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-04-21 22:52 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -7830,7 +7830,9 @@
         <v>0.25</v>
       </c>
       <c r="BZ11" s="12" t="n"/>
-      <c r="CA11" s="12" t="n"/>
+      <c r="CA11" s="12" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CB11" s="12" t="n"/>
       <c r="CC11" s="12" t="n"/>
       <c r="CD11" s="12" t="n"/>
@@ -10064,7 +10066,9 @@
         <v>5.25</v>
       </c>
       <c r="BZ19" s="12" t="n"/>
-      <c r="CA19" s="12" t="n"/>
+      <c r="CA19" s="12" t="n">
+        <v>6</v>
+      </c>
       <c r="CB19" s="12" t="n"/>
       <c r="CC19" s="12" t="n"/>
       <c r="CD19" s="12" t="n"/>
@@ -19520,7 +19524,9 @@
         <v>0.25</v>
       </c>
       <c r="BZ53" s="21" t="n"/>
-      <c r="CA53" s="21" t="n"/>
+      <c r="CA53" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CB53" s="21" t="n"/>
       <c r="CC53" s="21" t="n"/>
       <c r="CD53" s="21" t="n"/>
@@ -20074,7 +20080,9 @@
       <c r="BX55" s="21" t="n"/>
       <c r="BY55" s="21" t="n"/>
       <c r="BZ55" s="21" t="n"/>
-      <c r="CA55" s="21" t="n"/>
+      <c r="CA55" s="21" t="n">
+        <v>1.25</v>
+      </c>
       <c r="CB55" s="21" t="n"/>
       <c r="CC55" s="21" t="n"/>
       <c r="CD55" s="21" t="n"/>
@@ -25976,7 +25984,9 @@
         <v>0.25</v>
       </c>
       <c r="BZ76" s="21" t="n"/>
-      <c r="CA76" s="21" t="n"/>
+      <c r="CA76" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CB76" s="21" t="n"/>
       <c r="CC76" s="21" t="n"/>
       <c r="CD76" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-04-21 22:54 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -7833,7 +7833,9 @@
       <c r="CA11" s="12" t="n">
         <v>0.25</v>
       </c>
-      <c r="CB11" s="12" t="n"/>
+      <c r="CB11" s="12" t="n">
+        <v>1.25</v>
+      </c>
       <c r="CC11" s="12" t="n"/>
       <c r="CD11" s="12" t="n"/>
       <c r="CE11" s="12" t="n"/>
@@ -10069,7 +10071,9 @@
       <c r="CA19" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="CB19" s="12" t="n"/>
+      <c r="CB19" s="12" t="n">
+        <v>5.5</v>
+      </c>
       <c r="CC19" s="12" t="n"/>
       <c r="CD19" s="12" t="n"/>
       <c r="CE19" s="12" t="n"/>
@@ -17422,7 +17426,9 @@
       <c r="BY46" s="21" t="n"/>
       <c r="BZ46" s="21" t="n"/>
       <c r="CA46" s="21" t="n"/>
-      <c r="CB46" s="21" t="n"/>
+      <c r="CB46" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CC46" s="21" t="n"/>
       <c r="CD46" s="21" t="n"/>
       <c r="CE46" s="21" t="n"/>
@@ -18110,7 +18116,9 @@
       </c>
       <c r="BZ48" s="21" t="n"/>
       <c r="CA48" s="21" t="n"/>
-      <c r="CB48" s="21" t="n"/>
+      <c r="CB48" s="21" t="n">
+        <v>1</v>
+      </c>
       <c r="CC48" s="21" t="n"/>
       <c r="CD48" s="21" t="n"/>
       <c r="CE48" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-04-27 22:12 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -7837,7 +7837,9 @@
         <v>1.25</v>
       </c>
       <c r="CC11" s="12" t="n"/>
-      <c r="CD11" s="12" t="n"/>
+      <c r="CD11" s="12" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CE11" s="12" t="n"/>
       <c r="CF11" s="12" t="n"/>
       <c r="CG11" s="12" t="n"/>
@@ -10075,7 +10077,9 @@
         <v>5.5</v>
       </c>
       <c r="CC19" s="12" t="n"/>
-      <c r="CD19" s="12" t="n"/>
+      <c r="CD19" s="12" t="n">
+        <v>4.5</v>
+      </c>
       <c r="CE19" s="12" t="n"/>
       <c r="CF19" s="12" t="n"/>
       <c r="CG19" s="12" t="n"/>
@@ -18120,7 +18124,9 @@
         <v>1</v>
       </c>
       <c r="CC48" s="21" t="n"/>
-      <c r="CD48" s="21" t="n"/>
+      <c r="CD48" s="21" t="n">
+        <v>1</v>
+      </c>
       <c r="CE48" s="21" t="n"/>
       <c r="CF48" s="21" t="n"/>
       <c r="CG48" s="21" t="n"/>
@@ -19537,7 +19543,9 @@
       </c>
       <c r="CB53" s="21" t="n"/>
       <c r="CC53" s="21" t="n"/>
-      <c r="CD53" s="21" t="n"/>
+      <c r="CD53" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CE53" s="21" t="n"/>
       <c r="CF53" s="21" t="n"/>
       <c r="CG53" s="21" t="n"/>
@@ -24021,7 +24029,9 @@
       <c r="CA69" s="21" t="n"/>
       <c r="CB69" s="21" t="n"/>
       <c r="CC69" s="21" t="n"/>
-      <c r="CD69" s="21" t="n"/>
+      <c r="CD69" s="21" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CE69" s="21" t="n"/>
       <c r="CF69" s="21" t="n"/>
       <c r="CG69" s="21" t="n"/>
@@ -24293,7 +24303,9 @@
       <c r="CA70" s="21" t="n"/>
       <c r="CB70" s="21" t="n"/>
       <c r="CC70" s="21" t="n"/>
-      <c r="CD70" s="21" t="n"/>
+      <c r="CD70" s="21" t="n">
+        <v>0.75</v>
+      </c>
       <c r="CE70" s="21" t="n"/>
       <c r="CF70" s="21" t="n"/>
       <c r="CG70" s="21" t="n"/>
@@ -24826,7 +24838,9 @@
       <c r="CA72" s="21" t="n"/>
       <c r="CB72" s="21" t="n"/>
       <c r="CC72" s="21" t="n"/>
-      <c r="CD72" s="21" t="n"/>
+      <c r="CD72" s="21" t="n">
+        <v>0.75</v>
+      </c>
       <c r="CE72" s="21" t="n"/>
       <c r="CF72" s="21" t="n"/>
       <c r="CG72" s="21" t="n"/>
@@ -25997,7 +26011,9 @@
       </c>
       <c r="CB76" s="21" t="n"/>
       <c r="CC76" s="21" t="n"/>
-      <c r="CD76" s="21" t="n"/>
+      <c r="CD76" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CE76" s="21" t="n"/>
       <c r="CF76" s="21" t="n"/>
       <c r="CG76" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-04-27 22:13 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -7836,7 +7836,9 @@
       <c r="CB11" s="12" t="n">
         <v>1.25</v>
       </c>
-      <c r="CC11" s="12" t="n"/>
+      <c r="CC11" s="12" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CD11" s="12" t="n">
         <v>0.25</v>
       </c>
@@ -10076,7 +10078,9 @@
       <c r="CB19" s="12" t="n">
         <v>5.5</v>
       </c>
-      <c r="CC19" s="12" t="n"/>
+      <c r="CC19" s="12" t="n">
+        <v>5.25</v>
+      </c>
       <c r="CD19" s="12" t="n">
         <v>4.5</v>
       </c>
@@ -11440,7 +11444,9 @@
       <c r="BZ24" s="12" t="n"/>
       <c r="CA24" s="12" t="n"/>
       <c r="CB24" s="12" t="n"/>
-      <c r="CC24" s="12" t="n"/>
+      <c r="CC24" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="CD24" s="12" t="n"/>
       <c r="CE24" s="12" t="n"/>
       <c r="CF24" s="12" t="n"/>
@@ -17433,7 +17439,9 @@
       <c r="CB46" s="21" t="n">
         <v>0.25</v>
       </c>
-      <c r="CC46" s="21" t="n"/>
+      <c r="CC46" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CD46" s="21" t="n"/>
       <c r="CE46" s="21" t="n"/>
       <c r="CF46" s="21" t="n"/>
@@ -18123,7 +18131,9 @@
       <c r="CB48" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="CC48" s="21" t="n"/>
+      <c r="CC48" s="21" t="n">
+        <v>1</v>
+      </c>
       <c r="CD48" s="21" t="n">
         <v>1</v>
       </c>
@@ -19542,7 +19552,9 @@
         <v>0.25</v>
       </c>
       <c r="CB53" s="21" t="n"/>
-      <c r="CC53" s="21" t="n"/>
+      <c r="CC53" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CD53" s="21" t="n">
         <v>0.25</v>
       </c>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-04-27 22:15 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -9484,7 +9484,9 @@
       <c r="CB17" s="12" t="n"/>
       <c r="CC17" s="12" t="n"/>
       <c r="CD17" s="12" t="n"/>
-      <c r="CE17" s="12" t="n"/>
+      <c r="CE17" s="12" t="n">
+        <v>6.75</v>
+      </c>
       <c r="CF17" s="12" t="n"/>
       <c r="CG17" s="12" t="n"/>
       <c r="CH17" s="12" t="n"/>
@@ -18137,7 +18139,9 @@
       <c r="CD48" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="CE48" s="21" t="n"/>
+      <c r="CE48" s="21" t="n">
+        <v>1.25</v>
+      </c>
       <c r="CF48" s="21" t="n"/>
       <c r="CG48" s="21" t="n"/>
       <c r="CH48" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-04-27 22:17 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -10087,7 +10087,9 @@
         <v>4.5</v>
       </c>
       <c r="CE19" s="12" t="n"/>
-      <c r="CF19" s="12" t="n"/>
+      <c r="CF19" s="12" t="n">
+        <v>6.75</v>
+      </c>
       <c r="CG19" s="12" t="n"/>
       <c r="CH19" s="12" t="n"/>
       <c r="CI19" s="12" t="n"/>
@@ -18142,7 +18144,9 @@
       <c r="CE48" s="21" t="n">
         <v>1.25</v>
       </c>
-      <c r="CF48" s="21" t="n"/>
+      <c r="CF48" s="21" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CG48" s="21" t="n"/>
       <c r="CH48" s="21" t="n"/>
       <c r="CI48" s="21" t="n"/>
@@ -19563,7 +19567,9 @@
         <v>0.25</v>
       </c>
       <c r="CE53" s="21" t="n"/>
-      <c r="CF53" s="21" t="n"/>
+      <c r="CF53" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CG53" s="21" t="n"/>
       <c r="CH53" s="21" t="n"/>
       <c r="CI53" s="21" t="n"/>
@@ -20119,7 +20125,9 @@
       <c r="CC55" s="21" t="n"/>
       <c r="CD55" s="21" t="n"/>
       <c r="CE55" s="21" t="n"/>
-      <c r="CF55" s="21" t="n"/>
+      <c r="CF55" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CG55" s="21" t="n"/>
       <c r="CH55" s="21" t="n"/>
       <c r="CI55" s="21" t="n"/>
@@ -26031,7 +26039,9 @@
         <v>0.25</v>
       </c>
       <c r="CE76" s="21" t="n"/>
-      <c r="CF76" s="21" t="n"/>
+      <c r="CF76" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CG76" s="21" t="n"/>
       <c r="CH76" s="21" t="n"/>
       <c r="CI76" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-04-27 22:18 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -7844,7 +7844,9 @@
       </c>
       <c r="CE11" s="12" t="n"/>
       <c r="CF11" s="12" t="n"/>
-      <c r="CG11" s="12" t="n"/>
+      <c r="CG11" s="12" t="n">
+        <v>1.25</v>
+      </c>
       <c r="CH11" s="12" t="n"/>
       <c r="CI11" s="12" t="n"/>
       <c r="CJ11" s="19" t="n"/>
@@ -10090,7 +10092,9 @@
       <c r="CF19" s="12" t="n">
         <v>6.75</v>
       </c>
-      <c r="CG19" s="12" t="n"/>
+      <c r="CG19" s="12" t="n">
+        <v>6</v>
+      </c>
       <c r="CH19" s="12" t="n"/>
       <c r="CI19" s="12" t="n"/>
       <c r="CJ19" s="19" t="n"/>
@@ -17449,7 +17453,9 @@
       <c r="CD46" s="21" t="n"/>
       <c r="CE46" s="21" t="n"/>
       <c r="CF46" s="21" t="n"/>
-      <c r="CG46" s="21" t="n"/>
+      <c r="CG46" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CH46" s="21" t="n"/>
       <c r="CI46" s="21" t="n"/>
       <c r="CJ46" s="24" t="n"/>
@@ -26042,7 +26048,9 @@
       <c r="CF76" s="21" t="n">
         <v>0.25</v>
       </c>
-      <c r="CG76" s="21" t="n"/>
+      <c r="CG76" s="21" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CH76" s="21" t="n"/>
       <c r="CI76" s="21" t="n"/>
       <c r="CJ76" s="24" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-04-27 22:20 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -10083,7 +10083,7 @@
         <v>5.5</v>
       </c>
       <c r="CC19" s="12" t="n">
-        <v>5.25</v>
+        <v>3</v>
       </c>
       <c r="CD19" s="12" t="n">
         <v>4.5</v>
@@ -17448,7 +17448,7 @@
         <v>0.25</v>
       </c>
       <c r="CC46" s="21" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="CD46" s="21" t="n"/>
       <c r="CE46" s="21" t="n"/>
@@ -20128,7 +20128,9 @@
         <v>1.25</v>
       </c>
       <c r="CB55" s="21" t="n"/>
-      <c r="CC55" s="21" t="n"/>
+      <c r="CC55" s="21" t="n">
+        <v>2</v>
+      </c>
       <c r="CD55" s="21" t="n"/>
       <c r="CE55" s="21" t="n"/>
       <c r="CF55" s="21" t="n">

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-04-28 15:18 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -10093,7 +10093,7 @@
         <v>6.75</v>
       </c>
       <c r="CG19" s="12" t="n">
-        <v>6</v>
+        <v>5.75</v>
       </c>
       <c r="CH19" s="12" t="n"/>
       <c r="CI19" s="12" t="n"/>
@@ -11458,7 +11458,9 @@
       <c r="CD24" s="12" t="n"/>
       <c r="CE24" s="12" t="n"/>
       <c r="CF24" s="12" t="n"/>
-      <c r="CG24" s="12" t="n"/>
+      <c r="CG24" s="12" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CH24" s="12" t="n"/>
       <c r="CI24" s="12" t="n"/>
       <c r="CJ24" s="19" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-04-29 23:01 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -7848,7 +7848,9 @@
         <v>1.25</v>
       </c>
       <c r="CH11" s="12" t="n"/>
-      <c r="CI11" s="12" t="n"/>
+      <c r="CI11" s="12" t="n">
+        <v>1.25</v>
+      </c>
       <c r="CJ11" s="19" t="n"/>
       <c r="CK11" s="12" t="n"/>
       <c r="CL11" s="12" t="n"/>
@@ -8946,7 +8948,9 @@
       <c r="CF15" s="12" t="n"/>
       <c r="CG15" s="12" t="n"/>
       <c r="CH15" s="12" t="n"/>
-      <c r="CI15" s="12" t="n"/>
+      <c r="CI15" s="12" t="n">
+        <v>4</v>
+      </c>
       <c r="CJ15" s="19" t="n"/>
       <c r="CK15" s="12" t="n"/>
       <c r="CL15" s="12" t="n"/>
@@ -17459,7 +17463,9 @@
         <v>0.25</v>
       </c>
       <c r="CH46" s="21" t="n"/>
-      <c r="CI46" s="21" t="n"/>
+      <c r="CI46" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CJ46" s="24" t="n"/>
       <c r="CK46" s="21" t="n"/>
       <c r="CL46" s="21" t="n"/>
@@ -22864,7 +22870,9 @@
       <c r="CF65" s="21" t="n"/>
       <c r="CG65" s="21" t="n"/>
       <c r="CH65" s="21" t="n"/>
-      <c r="CI65" s="21" t="n"/>
+      <c r="CI65" s="21" t="n">
+        <v>2.25</v>
+      </c>
       <c r="CJ65" s="24" t="n"/>
       <c r="CK65" s="21" t="n"/>
       <c r="CL65" s="21" t="n"/>
@@ -23784,7 +23792,9 @@
       <c r="CF68" s="21" t="n"/>
       <c r="CG68" s="21" t="n"/>
       <c r="CH68" s="21" t="n"/>
-      <c r="CI68" s="21" t="n"/>
+      <c r="CI68" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CJ68" s="24" t="n"/>
       <c r="CK68" s="21" t="n"/>
       <c r="CL68" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-04-29 23:02 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -19586,7 +19586,9 @@
       </c>
       <c r="CG53" s="21" t="n"/>
       <c r="CH53" s="21" t="n"/>
-      <c r="CI53" s="21" t="n"/>
+      <c r="CI53" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CJ53" s="24" t="n"/>
       <c r="CK53" s="21" t="n"/>
       <c r="CL53" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-04-30 22:45 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -7851,7 +7851,9 @@
       <c r="CI11" s="12" t="n">
         <v>1.25</v>
       </c>
-      <c r="CJ11" s="19" t="n"/>
+      <c r="CJ11" s="19" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CK11" s="12" t="n"/>
       <c r="CL11" s="12" t="n"/>
       <c r="CM11" s="12" t="n"/>
@@ -8139,7 +8141,9 @@
       <c r="CG12" s="12" t="n"/>
       <c r="CH12" s="12" t="n"/>
       <c r="CI12" s="12" t="n"/>
-      <c r="CJ12" s="19" t="n"/>
+      <c r="CJ12" s="19" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CK12" s="12" t="n"/>
       <c r="CL12" s="12" t="n"/>
       <c r="CM12" s="12" t="n"/>
@@ -17466,7 +17470,9 @@
       <c r="CI46" s="21" t="n">
         <v>0.25</v>
       </c>
-      <c r="CJ46" s="24" t="n"/>
+      <c r="CJ46" s="24" t="n">
+        <v>2</v>
+      </c>
       <c r="CK46" s="21" t="n"/>
       <c r="CL46" s="21" t="n"/>
       <c r="CM46" s="21" t="n"/>
@@ -19589,7 +19595,9 @@
       <c r="CI53" s="21" t="n">
         <v>0.25</v>
       </c>
-      <c r="CJ53" s="24" t="n"/>
+      <c r="CJ53" s="24" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CK53" s="21" t="n"/>
       <c r="CL53" s="21" t="n"/>
       <c r="CM53" s="21" t="n"/>
@@ -22875,7 +22883,9 @@
       <c r="CI65" s="21" t="n">
         <v>2.25</v>
       </c>
-      <c r="CJ65" s="24" t="n"/>
+      <c r="CJ65" s="24" t="n">
+        <v>2</v>
+      </c>
       <c r="CK65" s="21" t="n"/>
       <c r="CL65" s="21" t="n"/>
       <c r="CM65" s="21" t="n"/>
@@ -23147,7 +23157,9 @@
       <c r="CG66" s="21" t="n"/>
       <c r="CH66" s="21" t="n"/>
       <c r="CI66" s="21" t="n"/>
-      <c r="CJ66" s="24" t="n"/>
+      <c r="CJ66" s="24" t="n">
+        <v>1.25</v>
+      </c>
       <c r="CK66" s="21" t="n"/>
       <c r="CL66" s="21" t="n"/>
       <c r="CM66" s="21" t="n"/>
@@ -23797,7 +23809,9 @@
       <c r="CI68" s="21" t="n">
         <v>0.25</v>
       </c>
-      <c r="CJ68" s="24" t="n"/>
+      <c r="CJ68" s="24" t="n">
+        <v>1.5</v>
+      </c>
       <c r="CK68" s="21" t="n"/>
       <c r="CL68" s="21" t="n"/>
       <c r="CM68" s="21" t="n"/>
@@ -26069,7 +26083,9 @@
       </c>
       <c r="CH76" s="21" t="n"/>
       <c r="CI76" s="21" t="n"/>
-      <c r="CJ76" s="24" t="n"/>
+      <c r="CJ76" s="24" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CK76" s="21" t="n"/>
       <c r="CL76" s="21" t="n"/>
       <c r="CM76" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-05-07 02:56 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -7854,7 +7854,9 @@
       <c r="CJ11" s="19" t="n">
         <v>0.25</v>
       </c>
-      <c r="CK11" s="12" t="n"/>
+      <c r="CK11" s="12" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CL11" s="12" t="n"/>
       <c r="CM11" s="12" t="n"/>
       <c r="CN11" s="12" t="n"/>
@@ -18171,7 +18173,9 @@
       <c r="CH48" s="21" t="n"/>
       <c r="CI48" s="21" t="n"/>
       <c r="CJ48" s="24" t="n"/>
-      <c r="CK48" s="21" t="n"/>
+      <c r="CK48" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CL48" s="21" t="n"/>
       <c r="CM48" s="21" t="n"/>
       <c r="CN48" s="21" t="n"/>
@@ -19598,7 +19602,9 @@
       <c r="CJ53" s="24" t="n">
         <v>0.25</v>
       </c>
-      <c r="CK53" s="21" t="n"/>
+      <c r="CK53" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CL53" s="21" t="n"/>
       <c r="CM53" s="21" t="n"/>
       <c r="CN53" s="21" t="n"/>
@@ -20158,7 +20164,9 @@
       <c r="CH55" s="21" t="n"/>
       <c r="CI55" s="21" t="n"/>
       <c r="CJ55" s="24" t="n"/>
-      <c r="CK55" s="21" t="n"/>
+      <c r="CK55" s="21" t="n">
+        <v>2</v>
+      </c>
       <c r="CL55" s="21" t="n"/>
       <c r="CM55" s="21" t="n"/>
       <c r="CN55" s="21" t="n"/>
@@ -24907,7 +24915,9 @@
       <c r="CH72" s="21" t="n"/>
       <c r="CI72" s="21" t="n"/>
       <c r="CJ72" s="24" t="n"/>
-      <c r="CK72" s="21" t="n"/>
+      <c r="CK72" s="21" t="n">
+        <v>5</v>
+      </c>
       <c r="CL72" s="21" t="n"/>
       <c r="CM72" s="21" t="n"/>
       <c r="CN72" s="21" t="n"/>
@@ -26086,7 +26096,9 @@
       <c r="CJ76" s="24" t="n">
         <v>0.25</v>
       </c>
-      <c r="CK76" s="21" t="n"/>
+      <c r="CK76" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CL76" s="21" t="n"/>
       <c r="CM76" s="21" t="n"/>
       <c r="CN76" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-05-07 22:13 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -7857,7 +7857,9 @@
       <c r="CK11" s="12" t="n">
         <v>0.25</v>
       </c>
-      <c r="CL11" s="12" t="n"/>
+      <c r="CL11" s="12" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CM11" s="12" t="n"/>
       <c r="CN11" s="12" t="n"/>
       <c r="CO11" s="12" t="n"/>
@@ -17476,7 +17478,9 @@
         <v>2</v>
       </c>
       <c r="CK46" s="21" t="n"/>
-      <c r="CL46" s="21" t="n"/>
+      <c r="CL46" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CM46" s="21" t="n"/>
       <c r="CN46" s="21" t="n"/>
       <c r="CO46" s="21" t="n"/>
@@ -18176,7 +18180,9 @@
       <c r="CK48" s="21" t="n">
         <v>0.25</v>
       </c>
-      <c r="CL48" s="21" t="n"/>
+      <c r="CL48" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CM48" s="21" t="n"/>
       <c r="CN48" s="21" t="n"/>
       <c r="CO48" s="21" t="n"/>
@@ -23821,7 +23827,9 @@
         <v>1.5</v>
       </c>
       <c r="CK68" s="21" t="n"/>
-      <c r="CL68" s="21" t="n"/>
+      <c r="CL68" s="21" t="n">
+        <v>2</v>
+      </c>
       <c r="CM68" s="21" t="n"/>
       <c r="CN68" s="21" t="n"/>
       <c r="CO68" s="21" t="n"/>
@@ -24918,7 +24926,9 @@
       <c r="CK72" s="21" t="n">
         <v>5</v>
       </c>
-      <c r="CL72" s="21" t="n"/>
+      <c r="CL72" s="21" t="n">
+        <v>5.25</v>
+      </c>
       <c r="CM72" s="21" t="n"/>
       <c r="CN72" s="21" t="n"/>
       <c r="CO72" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-05-07 22:16 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -18183,7 +18183,9 @@
       <c r="CL48" s="21" t="n">
         <v>0.25</v>
       </c>
-      <c r="CM48" s="21" t="n"/>
+      <c r="CM48" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CN48" s="21" t="n"/>
       <c r="CO48" s="21" t="n"/>
       <c r="CP48" s="21" t="n"/>
@@ -23470,7 +23472,9 @@
       <c r="CJ67" s="24" t="n"/>
       <c r="CK67" s="21" t="n"/>
       <c r="CL67" s="21" t="n"/>
-      <c r="CM67" s="21" t="n"/>
+      <c r="CM67" s="21" t="n">
+        <v>2.5</v>
+      </c>
       <c r="CN67" s="21" t="n"/>
       <c r="CO67" s="21" t="n"/>
       <c r="CP67" s="21" t="n"/>
@@ -24929,7 +24933,9 @@
       <c r="CL72" s="21" t="n">
         <v>5.25</v>
       </c>
-      <c r="CM72" s="21" t="n"/>
+      <c r="CM72" s="21" t="n">
+        <v>5.25</v>
+      </c>
       <c r="CN72" s="21" t="n"/>
       <c r="CO72" s="21" t="n"/>
       <c r="CP72" s="21" t="n"/>
@@ -26110,7 +26116,9 @@
         <v>0.25</v>
       </c>
       <c r="CL76" s="21" t="n"/>
-      <c r="CM76" s="21" t="n"/>
+      <c r="CM76" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CN76" s="21" t="n"/>
       <c r="CO76" s="21" t="n"/>
       <c r="CP76" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-05-07 22:18 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -7861,7 +7861,9 @@
         <v>0.25</v>
       </c>
       <c r="CM11" s="12" t="n"/>
-      <c r="CN11" s="12" t="n"/>
+      <c r="CN11" s="12" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CO11" s="12" t="n"/>
       <c r="CP11" s="12" t="n"/>
       <c r="CQ11" s="12" t="n"/>
@@ -17482,7 +17484,9 @@
         <v>0.25</v>
       </c>
       <c r="CM46" s="21" t="n"/>
-      <c r="CN46" s="21" t="n"/>
+      <c r="CN46" s="21" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CO46" s="21" t="n"/>
       <c r="CP46" s="21" t="n"/>
       <c r="CQ46" s="21" t="n"/>
@@ -18186,7 +18190,9 @@
       <c r="CM48" s="21" t="n">
         <v>0.25</v>
       </c>
-      <c r="CN48" s="21" t="n"/>
+      <c r="CN48" s="21" t="n">
+        <v>1.25</v>
+      </c>
       <c r="CO48" s="21" t="n"/>
       <c r="CP48" s="21" t="n"/>
       <c r="CQ48" s="21" t="n"/>
@@ -23835,7 +23841,9 @@
         <v>2</v>
       </c>
       <c r="CM68" s="21" t="n"/>
-      <c r="CN68" s="21" t="n"/>
+      <c r="CN68" s="21" t="n">
+        <v>1.5</v>
+      </c>
       <c r="CO68" s="21" t="n"/>
       <c r="CP68" s="21" t="n"/>
       <c r="CQ68" s="21" t="n"/>
@@ -26119,7 +26127,9 @@
       <c r="CM76" s="21" t="n">
         <v>0.25</v>
       </c>
-      <c r="CN76" s="21" t="n"/>
+      <c r="CN76" s="21" t="n">
+        <v>5.75</v>
+      </c>
       <c r="CO76" s="21" t="n"/>
       <c r="CP76" s="21" t="n"/>
       <c r="CQ76" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-05-07 22:21 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -7864,7 +7864,9 @@
       <c r="CN11" s="12" t="n">
         <v>0.25</v>
       </c>
-      <c r="CO11" s="12" t="n"/>
+      <c r="CO11" s="12" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CP11" s="12" t="n"/>
       <c r="CQ11" s="12" t="n"/>
       <c r="CR11" s="12" t="n"/>
@@ -8154,7 +8156,9 @@
       <c r="CL12" s="12" t="n"/>
       <c r="CM12" s="12" t="n"/>
       <c r="CN12" s="12" t="n"/>
-      <c r="CO12" s="12" t="n"/>
+      <c r="CO12" s="12" t="n">
+        <v>0.75</v>
+      </c>
       <c r="CP12" s="12" t="n"/>
       <c r="CQ12" s="12" t="n"/>
       <c r="CR12" s="12" t="n"/>
@@ -17487,7 +17491,9 @@
       <c r="CN46" s="21" t="n">
         <v>0.5</v>
       </c>
-      <c r="CO46" s="21" t="n"/>
+      <c r="CO46" s="21" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CP46" s="21" t="n"/>
       <c r="CQ46" s="21" t="n"/>
       <c r="CR46" s="21" t="n"/>
@@ -18193,7 +18199,9 @@
       <c r="CN48" s="21" t="n">
         <v>1.25</v>
       </c>
-      <c r="CO48" s="21" t="n"/>
+      <c r="CO48" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CP48" s="21" t="n"/>
       <c r="CQ48" s="21" t="n"/>
       <c r="CR48" s="21" t="n"/>
@@ -19622,7 +19630,9 @@
       <c r="CL53" s="21" t="n"/>
       <c r="CM53" s="21" t="n"/>
       <c r="CN53" s="21" t="n"/>
-      <c r="CO53" s="21" t="n"/>
+      <c r="CO53" s="21" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CP53" s="21" t="n"/>
       <c r="CQ53" s="21" t="n"/>
       <c r="CR53" s="21" t="n"/>
@@ -23844,7 +23854,9 @@
       <c r="CN68" s="21" t="n">
         <v>1.5</v>
       </c>
-      <c r="CO68" s="21" t="n"/>
+      <c r="CO68" s="21" t="n">
+        <v>2</v>
+      </c>
       <c r="CP68" s="21" t="n"/>
       <c r="CQ68" s="21" t="n"/>
       <c r="CR68" s="21" t="n"/>
@@ -24945,7 +24957,9 @@
         <v>5.25</v>
       </c>
       <c r="CN72" s="21" t="n"/>
-      <c r="CO72" s="21" t="n"/>
+      <c r="CO72" s="21" t="n">
+        <v>3.5</v>
+      </c>
       <c r="CP72" s="21" t="n"/>
       <c r="CQ72" s="21" t="n"/>
       <c r="CR72" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-05-11 22:26 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -23196,7 +23196,9 @@
       <c r="CL66" s="21" t="n"/>
       <c r="CM66" s="21" t="n"/>
       <c r="CN66" s="21" t="n"/>
-      <c r="CO66" s="21" t="n"/>
+      <c r="CO66" s="21" t="n">
+        <v>3</v>
+      </c>
       <c r="CP66" s="21" t="n"/>
       <c r="CQ66" s="21" t="n"/>
       <c r="CR66" s="21" t="n"/>
@@ -24957,9 +24959,7 @@
         <v>5.25</v>
       </c>
       <c r="CN72" s="21" t="n"/>
-      <c r="CO72" s="21" t="n">
-        <v>3.5</v>
-      </c>
+      <c r="CO72" s="21" t="n"/>
       <c r="CP72" s="21" t="n"/>
       <c r="CQ72" s="21" t="n"/>
       <c r="CR72" s="21" t="n"/>
@@ -26694,7 +26694,9 @@
       <c r="CL78" s="21" t="n"/>
       <c r="CM78" s="21" t="n"/>
       <c r="CN78" s="21" t="n"/>
-      <c r="CO78" s="21" t="n"/>
+      <c r="CO78" s="21" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CP78" s="21" t="n"/>
       <c r="CQ78" s="21" t="n"/>
       <c r="CR78" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-05-11 22:27 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -24949,9 +24949,7 @@
       <c r="CH72" s="21" t="n"/>
       <c r="CI72" s="21" t="n"/>
       <c r="CJ72" s="24" t="n"/>
-      <c r="CK72" s="21" t="n">
-        <v>5</v>
-      </c>
+      <c r="CK72" s="21" t="n"/>
       <c r="CL72" s="21" t="n">
         <v>5.25</v>
       </c>
@@ -26690,7 +26688,9 @@
       <c r="CH78" s="21" t="n"/>
       <c r="CI78" s="21" t="n"/>
       <c r="CJ78" s="24" t="n"/>
-      <c r="CK78" s="21" t="n"/>
+      <c r="CK78" s="21" t="n">
+        <v>5</v>
+      </c>
       <c r="CL78" s="21" t="n"/>
       <c r="CM78" s="21" t="n"/>
       <c r="CN78" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-05-11 22:31 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -10113,7 +10113,9 @@
       <c r="CG19" s="12" t="n">
         <v>5.75</v>
       </c>
-      <c r="CH19" s="12" t="n"/>
+      <c r="CH19" s="12" t="n">
+        <v>7.25</v>
+      </c>
       <c r="CI19" s="12" t="n"/>
       <c r="CJ19" s="19" t="n"/>
       <c r="CK19" s="12" t="n"/>
@@ -18184,7 +18186,9 @@
         <v>0.5</v>
       </c>
       <c r="CG48" s="21" t="n"/>
-      <c r="CH48" s="21" t="n"/>
+      <c r="CH48" s="21" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CI48" s="21" t="n"/>
       <c r="CJ48" s="24" t="n"/>
       <c r="CK48" s="21" t="n">
@@ -26127,7 +26131,9 @@
       <c r="CG76" s="21" t="n">
         <v>0.5</v>
       </c>
-      <c r="CH76" s="21" t="n"/>
+      <c r="CH76" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CI76" s="21" t="n"/>
       <c r="CJ76" s="24" t="n">
         <v>0.25</v>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-05-11 22:32 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -24954,9 +24954,7 @@
       <c r="CI72" s="21" t="n"/>
       <c r="CJ72" s="24" t="n"/>
       <c r="CK72" s="21" t="n"/>
-      <c r="CL72" s="21" t="n">
-        <v>5.25</v>
-      </c>
+      <c r="CL72" s="21" t="n"/>
       <c r="CM72" s="21" t="n">
         <v>5.25</v>
       </c>
@@ -26697,7 +26695,9 @@
       <c r="CK78" s="21" t="n">
         <v>5</v>
       </c>
-      <c r="CL78" s="21" t="n"/>
+      <c r="CL78" s="21" t="n">
+        <v>5.25</v>
+      </c>
       <c r="CM78" s="21" t="n"/>
       <c r="CN78" s="21" t="n"/>
       <c r="CO78" s="21" t="n">

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-05-11 22:33 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -26142,7 +26142,7 @@
         <v>0.25</v>
       </c>
       <c r="CN76" s="21" t="n">
-        <v>5.75</v>
+        <v>0.25</v>
       </c>
       <c r="CO76" s="21" t="n"/>
       <c r="CP76" s="21" t="n"/>
@@ -26699,7 +26699,9 @@
       <c r="CM78" s="21" t="n">
         <v>5.25</v>
       </c>
-      <c r="CN78" s="21" t="n"/>
+      <c r="CN78" s="21" t="n">
+        <v>5.5</v>
+      </c>
       <c r="CO78" s="21" t="n">
         <v>0.5</v>
       </c>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-05-11 22:35 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -7867,7 +7867,9 @@
       <c r="CO11" s="12" t="n">
         <v>0.5</v>
       </c>
-      <c r="CP11" s="12" t="n"/>
+      <c r="CP11" s="12" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CQ11" s="12" t="n"/>
       <c r="CR11" s="12" t="n"/>
       <c r="CS11" s="12" t="n"/>
@@ -17496,7 +17498,9 @@
       <c r="CO46" s="21" t="n">
         <v>0.5</v>
       </c>
-      <c r="CP46" s="21" t="n"/>
+      <c r="CP46" s="21" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CQ46" s="21" t="n"/>
       <c r="CR46" s="21" t="n"/>
       <c r="CS46" s="21" t="n"/>
@@ -18206,7 +18210,9 @@
       <c r="CO48" s="21" t="n">
         <v>0.25</v>
       </c>
-      <c r="CP48" s="21" t="n"/>
+      <c r="CP48" s="21" t="n">
+        <v>5</v>
+      </c>
       <c r="CQ48" s="21" t="n"/>
       <c r="CR48" s="21" t="n"/>
       <c r="CS48" s="21" t="n"/>
@@ -23203,7 +23209,9 @@
       <c r="CO66" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="CP66" s="21" t="n"/>
+      <c r="CP66" s="21" t="n">
+        <v>2.5</v>
+      </c>
       <c r="CQ66" s="21" t="n"/>
       <c r="CR66" s="21" t="n"/>
       <c r="CS66" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-05-11 22:37 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -7870,7 +7870,9 @@
       <c r="CP11" s="12" t="n">
         <v>0.25</v>
       </c>
-      <c r="CQ11" s="12" t="n"/>
+      <c r="CQ11" s="12" t="n">
+        <v>1.75</v>
+      </c>
       <c r="CR11" s="12" t="n"/>
       <c r="CS11" s="12" t="n"/>
       <c r="CT11" s="12" t="n"/>
@@ -17501,7 +17503,9 @@
       <c r="CP46" s="21" t="n">
         <v>0.5</v>
       </c>
-      <c r="CQ46" s="21" t="n"/>
+      <c r="CQ46" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CR46" s="21" t="n"/>
       <c r="CS46" s="21" t="n"/>
       <c r="CT46" s="21" t="n"/>
@@ -18213,7 +18217,9 @@
       <c r="CP48" s="21" t="n">
         <v>5</v>
       </c>
-      <c r="CQ48" s="21" t="n"/>
+      <c r="CQ48" s="21" t="n">
+        <v>5.5</v>
+      </c>
       <c r="CR48" s="21" t="n"/>
       <c r="CS48" s="21" t="n"/>
       <c r="CT48" s="21" t="n"/>
@@ -19644,7 +19650,9 @@
         <v>0.5</v>
       </c>
       <c r="CP53" s="21" t="n"/>
-      <c r="CQ53" s="21" t="n"/>
+      <c r="CQ53" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CR53" s="21" t="n"/>
       <c r="CS53" s="21" t="n"/>
       <c r="CT53" s="21" t="n"/>
@@ -26154,7 +26162,9 @@
       </c>
       <c r="CO76" s="21" t="n"/>
       <c r="CP76" s="21" t="n"/>
-      <c r="CQ76" s="21" t="n"/>
+      <c r="CQ76" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CR76" s="21" t="n"/>
       <c r="CS76" s="21" t="n"/>
       <c r="CT76" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-05-12 22:20 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -7873,7 +7873,9 @@
       <c r="CQ11" s="12" t="n">
         <v>1.75</v>
       </c>
-      <c r="CR11" s="12" t="n"/>
+      <c r="CR11" s="12" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CS11" s="12" t="n"/>
       <c r="CT11" s="12" t="n"/>
       <c r="CU11" s="12" t="n"/>
@@ -17506,7 +17508,9 @@
       <c r="CQ46" s="21" t="n">
         <v>0.25</v>
       </c>
-      <c r="CR46" s="21" t="n"/>
+      <c r="CR46" s="21" t="n">
+        <v>0.75</v>
+      </c>
       <c r="CS46" s="21" t="n"/>
       <c r="CT46" s="21" t="n"/>
       <c r="CU46" s="21" t="n"/>
@@ -18220,7 +18224,9 @@
       <c r="CQ48" s="21" t="n">
         <v>5.5</v>
       </c>
-      <c r="CR48" s="21" t="n"/>
+      <c r="CR48" s="21" t="n">
+        <v>6.75</v>
+      </c>
       <c r="CS48" s="21" t="n"/>
       <c r="CT48" s="21" t="n"/>
       <c r="CU48" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-05-13 22:23 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -7876,7 +7876,9 @@
       <c r="CR11" s="12" t="n">
         <v>0.5</v>
       </c>
-      <c r="CS11" s="12" t="n"/>
+      <c r="CS11" s="12" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CT11" s="12" t="n"/>
       <c r="CU11" s="12" t="n"/>
       <c r="CV11" s="12" t="n"/>
@@ -8168,7 +8170,9 @@
       <c r="CP12" s="12" t="n"/>
       <c r="CQ12" s="12" t="n"/>
       <c r="CR12" s="12" t="n"/>
-      <c r="CS12" s="12" t="n"/>
+      <c r="CS12" s="12" t="n">
+        <v>0.75</v>
+      </c>
       <c r="CT12" s="12" t="n"/>
       <c r="CU12" s="12" t="n"/>
       <c r="CV12" s="12" t="n"/>
@@ -11498,7 +11502,9 @@
       <c r="CP24" s="12" t="n"/>
       <c r="CQ24" s="12" t="n"/>
       <c r="CR24" s="12" t="n"/>
-      <c r="CS24" s="12" t="n"/>
+      <c r="CS24" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="CT24" s="12" t="n"/>
       <c r="CU24" s="12" t="n"/>
       <c r="CV24" s="12" t="n"/>
@@ -17511,7 +17517,9 @@
       <c r="CR46" s="21" t="n">
         <v>0.75</v>
       </c>
-      <c r="CS46" s="21" t="n"/>
+      <c r="CS46" s="21" t="n">
+        <v>1.75</v>
+      </c>
       <c r="CT46" s="21" t="n"/>
       <c r="CU46" s="21" t="n"/>
       <c r="CV46" s="21" t="n"/>
@@ -18227,7 +18235,9 @@
       <c r="CR48" s="21" t="n">
         <v>6.75</v>
       </c>
-      <c r="CS48" s="21" t="n"/>
+      <c r="CS48" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CT48" s="21" t="n"/>
       <c r="CU48" s="21" t="n"/>
       <c r="CV48" s="21" t="n"/>
@@ -20222,7 +20232,9 @@
       <c r="CP55" s="21" t="n"/>
       <c r="CQ55" s="21" t="n"/>
       <c r="CR55" s="21" t="n"/>
-      <c r="CS55" s="21" t="n"/>
+      <c r="CS55" s="21" t="n">
+        <v>1.5</v>
+      </c>
       <c r="CT55" s="21" t="n"/>
       <c r="CU55" s="21" t="n"/>
       <c r="CV55" s="21" t="n"/>
@@ -26172,7 +26184,9 @@
         <v>0.25</v>
       </c>
       <c r="CR76" s="21" t="n"/>
-      <c r="CS76" s="21" t="n"/>
+      <c r="CS76" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CT76" s="21" t="n"/>
       <c r="CU76" s="21" t="n"/>
       <c r="CV76" s="21" t="n"/>
@@ -26450,7 +26464,9 @@
       <c r="CP77" s="21" t="n"/>
       <c r="CQ77" s="21" t="n"/>
       <c r="CR77" s="21" t="n"/>
-      <c r="CS77" s="21" t="n"/>
+      <c r="CS77" s="21" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CT77" s="21" t="n"/>
       <c r="CU77" s="21" t="n"/>
       <c r="CV77" s="21" t="n"/>
@@ -26732,7 +26748,9 @@
       <c r="CP78" s="21" t="n"/>
       <c r="CQ78" s="21" t="n"/>
       <c r="CR78" s="21" t="n"/>
-      <c r="CS78" s="21" t="n"/>
+      <c r="CS78" s="21" t="n">
+        <v>1.5</v>
+      </c>
       <c r="CT78" s="21" t="n"/>
       <c r="CU78" s="21" t="n"/>
       <c r="CV78" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-05-15 21:01 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -8173,7 +8173,9 @@
       <c r="CS12" s="12" t="n">
         <v>0.75</v>
       </c>
-      <c r="CT12" s="12" t="n"/>
+      <c r="CT12" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="CU12" s="12" t="n"/>
       <c r="CV12" s="12" t="n"/>
       <c r="CW12" s="12" t="n"/>
@@ -13961,7 +13963,9 @@
       <c r="CQ33" s="21" t="n"/>
       <c r="CR33" s="21" t="n"/>
       <c r="CS33" s="21" t="n"/>
-      <c r="CT33" s="21" t="n"/>
+      <c r="CT33" s="21" t="n">
+        <v>3</v>
+      </c>
       <c r="CU33" s="21" t="n"/>
       <c r="CV33" s="21" t="n"/>
       <c r="CW33" s="21" t="n"/>
@@ -17520,7 +17524,9 @@
       <c r="CS46" s="21" t="n">
         <v>1.75</v>
       </c>
-      <c r="CT46" s="21" t="n"/>
+      <c r="CT46" s="21" t="n">
+        <v>1.5</v>
+      </c>
       <c r="CU46" s="21" t="n"/>
       <c r="CV46" s="21" t="n"/>
       <c r="CW46" s="21" t="n"/>
@@ -18238,7 +18244,9 @@
       <c r="CS48" s="21" t="n">
         <v>0.25</v>
       </c>
-      <c r="CT48" s="21" t="n"/>
+      <c r="CT48" s="21" t="n">
+        <v>1.25</v>
+      </c>
       <c r="CU48" s="21" t="n"/>
       <c r="CV48" s="21" t="n"/>
       <c r="CW48" s="21" t="n"/>
@@ -20235,7 +20243,9 @@
       <c r="CS55" s="21" t="n">
         <v>1.5</v>
       </c>
-      <c r="CT55" s="21" t="n"/>
+      <c r="CT55" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CU55" s="21" t="n"/>
       <c r="CV55" s="21" t="n"/>
       <c r="CW55" s="21" t="n"/>
@@ -26187,7 +26197,9 @@
       <c r="CS76" s="21" t="n">
         <v>0.25</v>
       </c>
-      <c r="CT76" s="21" t="n"/>
+      <c r="CT76" s="21" t="n">
+        <v>1</v>
+      </c>
       <c r="CU76" s="21" t="n"/>
       <c r="CV76" s="21" t="n"/>
       <c r="CW76" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-05-15 21:03 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -13966,7 +13966,9 @@
       <c r="CT33" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="CU33" s="21" t="n"/>
+      <c r="CU33" s="21" t="n">
+        <v>2</v>
+      </c>
       <c r="CV33" s="21" t="n"/>
       <c r="CW33" s="21" t="n"/>
       <c r="CX33" s="21" t="n"/>
@@ -17527,7 +17529,9 @@
       <c r="CT46" s="21" t="n">
         <v>1.5</v>
       </c>
-      <c r="CU46" s="21" t="n"/>
+      <c r="CU46" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CV46" s="21" t="n"/>
       <c r="CW46" s="21" t="n"/>
       <c r="CX46" s="21" t="n"/>
@@ -18247,7 +18251,9 @@
       <c r="CT48" s="21" t="n">
         <v>1.25</v>
       </c>
-      <c r="CU48" s="21" t="n"/>
+      <c r="CU48" s="21" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CV48" s="21" t="n"/>
       <c r="CW48" s="21" t="n"/>
       <c r="CX48" s="21" t="n"/>
@@ -26200,7 +26206,9 @@
       <c r="CT76" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="CU76" s="21" t="n"/>
+      <c r="CU76" s="21" t="n">
+        <v>1.25</v>
+      </c>
       <c r="CV76" s="21" t="n"/>
       <c r="CW76" s="21" t="n"/>
       <c r="CX76" s="21" t="n"/>
@@ -28151,7 +28159,9 @@
       <c r="CR83" s="21" t="n"/>
       <c r="CS83" s="21" t="n"/>
       <c r="CT83" s="21" t="n"/>
-      <c r="CU83" s="21" t="n"/>
+      <c r="CU83" s="21" t="n">
+        <v>4</v>
+      </c>
       <c r="CV83" s="21" t="n"/>
       <c r="CW83" s="21" t="n"/>
       <c r="CX83" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-05-18 22:17 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -17532,7 +17532,9 @@
       <c r="CU46" s="21" t="n">
         <v>0.25</v>
       </c>
-      <c r="CV46" s="21" t="n"/>
+      <c r="CV46" s="21" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CW46" s="21" t="n"/>
       <c r="CX46" s="21" t="n"/>
       <c r="CY46" s="21" t="n"/>
@@ -18254,7 +18256,9 @@
       <c r="CU48" s="21" t="n">
         <v>0.5</v>
       </c>
-      <c r="CV48" s="21" t="n"/>
+      <c r="CV48" s="21" t="n">
+        <v>5.75</v>
+      </c>
       <c r="CW48" s="21" t="n"/>
       <c r="CX48" s="21" t="n"/>
       <c r="CY48" s="21" t="n"/>
@@ -19961,7 +19965,9 @@
       <c r="CS54" s="21" t="n"/>
       <c r="CT54" s="21" t="n"/>
       <c r="CU54" s="21" t="n"/>
-      <c r="CV54" s="21" t="n"/>
+      <c r="CV54" s="21" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CW54" s="21" t="n"/>
       <c r="CX54" s="21" t="n"/>
       <c r="CY54" s="21" t="n"/>
@@ -25014,7 +25020,9 @@
       <c r="CS72" s="21" t="n"/>
       <c r="CT72" s="21" t="n"/>
       <c r="CU72" s="21" t="n"/>
-      <c r="CV72" s="21" t="n"/>
+      <c r="CV72" s="21" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CW72" s="21" t="n"/>
       <c r="CX72" s="21" t="n"/>
       <c r="CY72" s="21" t="n"/>
@@ -26489,7 +26497,9 @@
       </c>
       <c r="CT77" s="21" t="n"/>
       <c r="CU77" s="21" t="n"/>
-      <c r="CV77" s="21" t="n"/>
+      <c r="CV77" s="21" t="n">
+        <v>0.75</v>
+      </c>
       <c r="CW77" s="21" t="n"/>
       <c r="CX77" s="21" t="n"/>
       <c r="CY77" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-05-18 22:18 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -19691,7 +19691,9 @@
       <c r="CS53" s="21" t="n"/>
       <c r="CT53" s="21" t="n"/>
       <c r="CU53" s="21" t="n"/>
-      <c r="CV53" s="21" t="n"/>
+      <c r="CV53" s="21" t="n">
+        <v>0.75</v>
+      </c>
       <c r="CW53" s="21" t="n"/>
       <c r="CX53" s="21" t="n"/>
       <c r="CY53" s="21" t="n"/>
@@ -19965,9 +19967,7 @@
       <c r="CS54" s="21" t="n"/>
       <c r="CT54" s="21" t="n"/>
       <c r="CU54" s="21" t="n"/>
-      <c r="CV54" s="21" t="n">
-        <v>0.5</v>
-      </c>
+      <c r="CV54" s="21" t="n"/>
       <c r="CW54" s="21" t="n"/>
       <c r="CX54" s="21" t="n"/>
       <c r="CY54" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-05-20 22:23 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -7882,7 +7882,9 @@
       <c r="CT11" s="12" t="n"/>
       <c r="CU11" s="12" t="n"/>
       <c r="CV11" s="12" t="n"/>
-      <c r="CW11" s="12" t="n"/>
+      <c r="CW11" s="12" t="n">
+        <v>1.25</v>
+      </c>
       <c r="CX11" s="12" t="n"/>
       <c r="CY11" s="12" t="n"/>
       <c r="CZ11" s="12" t="n"/>
@@ -17195,7 +17197,9 @@
       <c r="CT45" s="21" t="n"/>
       <c r="CU45" s="21" t="n"/>
       <c r="CV45" s="21" t="n"/>
-      <c r="CW45" s="21" t="n"/>
+      <c r="CW45" s="21" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CX45" s="21" t="n"/>
       <c r="CY45" s="21" t="n"/>
       <c r="CZ45" s="21" t="n"/>
@@ -18259,7 +18263,9 @@
       <c r="CV48" s="21" t="n">
         <v>5.75</v>
       </c>
-      <c r="CW48" s="21" t="n"/>
+      <c r="CW48" s="21" t="n">
+        <v>5</v>
+      </c>
       <c r="CX48" s="21" t="n"/>
       <c r="CY48" s="21" t="n"/>
       <c r="CZ48" s="21" t="n"/>
@@ -19694,7 +19700,9 @@
       <c r="CV53" s="21" t="n">
         <v>0.75</v>
       </c>
-      <c r="CW53" s="21" t="n"/>
+      <c r="CW53" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CX53" s="21" t="n"/>
       <c r="CY53" s="21" t="n"/>
       <c r="CZ53" s="21" t="n"/>
@@ -25023,7 +25031,9 @@
       <c r="CV72" s="21" t="n">
         <v>0.5</v>
       </c>
-      <c r="CW72" s="21" t="n"/>
+      <c r="CW72" s="21" t="n">
+        <v>0.75</v>
+      </c>
       <c r="CX72" s="21" t="n"/>
       <c r="CY72" s="21" t="n"/>
       <c r="CZ72" s="21" t="n"/>
@@ -26218,7 +26228,9 @@
         <v>1.25</v>
       </c>
       <c r="CV76" s="21" t="n"/>
-      <c r="CW76" s="21" t="n"/>
+      <c r="CW76" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CX76" s="21" t="n"/>
       <c r="CY76" s="21" t="n"/>
       <c r="CZ76" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-05-20 22:35 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -7885,7 +7885,9 @@
       <c r="CW11" s="12" t="n">
         <v>1.25</v>
       </c>
-      <c r="CX11" s="12" t="n"/>
+      <c r="CX11" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="CY11" s="12" t="n"/>
       <c r="CZ11" s="12" t="n"/>
       <c r="DA11" s="12" t="n"/>
@@ -13973,7 +13975,9 @@
       </c>
       <c r="CV33" s="21" t="n"/>
       <c r="CW33" s="21" t="n"/>
-      <c r="CX33" s="21" t="n"/>
+      <c r="CX33" s="21" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CY33" s="21" t="n"/>
       <c r="CZ33" s="21" t="n"/>
       <c r="DA33" s="21" t="n"/>
@@ -17540,7 +17544,9 @@
         <v>0.5</v>
       </c>
       <c r="CW46" s="21" t="n"/>
-      <c r="CX46" s="21" t="n"/>
+      <c r="CX46" s="21" t="n">
+        <v>2.5</v>
+      </c>
       <c r="CY46" s="21" t="n"/>
       <c r="CZ46" s="21" t="n"/>
       <c r="DA46" s="21" t="n"/>
@@ -18266,7 +18272,9 @@
       <c r="CW48" s="21" t="n">
         <v>5</v>
       </c>
-      <c r="CX48" s="21" t="n"/>
+      <c r="CX48" s="21" t="n">
+        <v>1.75</v>
+      </c>
       <c r="CY48" s="21" t="n"/>
       <c r="CZ48" s="21" t="n"/>
       <c r="DA48" s="21" t="n"/>
@@ -19977,7 +19985,9 @@
       <c r="CU54" s="21" t="n"/>
       <c r="CV54" s="21" t="n"/>
       <c r="CW54" s="21" t="n"/>
-      <c r="CX54" s="21" t="n"/>
+      <c r="CX54" s="21" t="n">
+        <v>0.5</v>
+      </c>
       <c r="CY54" s="21" t="n"/>
       <c r="CZ54" s="21" t="n"/>
       <c r="DA54" s="21" t="n"/>
@@ -26231,7 +26241,9 @@
       <c r="CW76" s="21" t="n">
         <v>0.25</v>
       </c>
-      <c r="CX76" s="21" t="n"/>
+      <c r="CX76" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="CY76" s="21" t="n"/>
       <c r="CZ76" s="21" t="n"/>
       <c r="DA76" s="21" t="n"/>
@@ -26797,7 +26809,9 @@
       <c r="CU78" s="21" t="n"/>
       <c r="CV78" s="21" t="n"/>
       <c r="CW78" s="21" t="n"/>
-      <c r="CX78" s="21" t="n"/>
+      <c r="CX78" s="21" t="n">
+        <v>1.5</v>
+      </c>
       <c r="CY78" s="21" t="n"/>
       <c r="CZ78" s="21" t="n"/>
       <c r="DA78" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-05-20 22:36 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -28204,7 +28204,9 @@
       <c r="CY83" s="21" t="n">
         <v>8</v>
       </c>
-      <c r="CZ83" s="21" t="n"/>
+      <c r="CZ83" s="21" t="n">
+        <v>8</v>
+      </c>
       <c r="DA83" s="21" t="n"/>
       <c r="DB83" s="21" t="n"/>
       <c r="DC83" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-05-20 22:38 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -27925,7 +27925,9 @@
       <c r="CY82" s="21" t="n"/>
       <c r="CZ82" s="21" t="n"/>
       <c r="DA82" s="21" t="n"/>
-      <c r="DB82" s="21" t="n"/>
+      <c r="DB82" s="21" t="n">
+        <v>8</v>
+      </c>
       <c r="DC82" s="21" t="n"/>
       <c r="DD82" s="21" t="n"/>
       <c r="DE82" s="24" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-05-20 22:39 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -27937,7 +27937,9 @@
       <c r="DE82" s="24" t="n">
         <v>8</v>
       </c>
-      <c r="DF82" s="21" t="n"/>
+      <c r="DF82" s="21" t="n">
+        <v>8</v>
+      </c>
       <c r="DG82" s="21" t="n"/>
       <c r="DH82" s="21" t="n"/>
       <c r="DI82" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-06-10 22:11 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -7902,7 +7902,9 @@
       <c r="DJ11" s="12" t="n"/>
       <c r="DK11" s="12" t="n"/>
       <c r="DL11" s="12" t="n"/>
-      <c r="DM11" s="12" t="n"/>
+      <c r="DM11" s="12" t="n">
+        <v>0.25</v>
+      </c>
       <c r="DN11" s="12" t="n"/>
       <c r="DO11" s="12" t="n"/>
       <c r="DP11" s="12" t="n"/>
@@ -13992,7 +13994,9 @@
       <c r="DJ33" s="21" t="n"/>
       <c r="DK33" s="21" t="n"/>
       <c r="DL33" s="21" t="n"/>
-      <c r="DM33" s="21" t="n"/>
+      <c r="DM33" s="21" t="n">
+        <v>6</v>
+      </c>
       <c r="DN33" s="21" t="n"/>
       <c r="DO33" s="21" t="n"/>
       <c r="DP33" s="21" t="n"/>
@@ -23300,7 +23304,9 @@
       <c r="DJ66" s="21" t="n"/>
       <c r="DK66" s="21" t="n"/>
       <c r="DL66" s="21" t="n"/>
-      <c r="DM66" s="21" t="n"/>
+      <c r="DM66" s="21" t="n">
+        <v>0.5</v>
+      </c>
       <c r="DN66" s="21" t="n"/>
       <c r="DO66" s="21" t="n"/>
       <c r="DP66" s="21" t="n"/>
@@ -23960,7 +23966,9 @@
       <c r="DJ68" s="21" t="n"/>
       <c r="DK68" s="21" t="n"/>
       <c r="DL68" s="21" t="n"/>
-      <c r="DM68" s="21" t="n"/>
+      <c r="DM68" s="21" t="n">
+        <v>0.5</v>
+      </c>
       <c r="DN68" s="21" t="n"/>
       <c r="DO68" s="21" t="n"/>
       <c r="DP68" s="21" t="n"/>
@@ -26258,7 +26266,9 @@
       <c r="DJ76" s="21" t="n"/>
       <c r="DK76" s="21" t="n"/>
       <c r="DL76" s="21" t="n"/>
-      <c r="DM76" s="21" t="n"/>
+      <c r="DM76" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="DN76" s="21" t="n"/>
       <c r="DO76" s="21" t="n"/>
       <c r="DP76" s="21" t="n"/>
@@ -26540,7 +26550,9 @@
       <c r="DJ77" s="21" t="n"/>
       <c r="DK77" s="21" t="n"/>
       <c r="DL77" s="21" t="n"/>
-      <c r="DM77" s="21" t="n"/>
+      <c r="DM77" s="21" t="n">
+        <v>0.5</v>
+      </c>
       <c r="DN77" s="21" t="n"/>
       <c r="DO77" s="21" t="n"/>
       <c r="DP77" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-06-10 22:13 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -13993,7 +13993,9 @@
       <c r="DI33" s="21" t="n"/>
       <c r="DJ33" s="21" t="n"/>
       <c r="DK33" s="21" t="n"/>
-      <c r="DL33" s="21" t="n"/>
+      <c r="DL33" s="21" t="n">
+        <v>6</v>
+      </c>
       <c r="DM33" s="21" t="n">
         <v>6</v>
       </c>
@@ -18292,7 +18294,9 @@
       <c r="DI48" s="21" t="n"/>
       <c r="DJ48" s="21" t="n"/>
       <c r="DK48" s="21" t="n"/>
-      <c r="DL48" s="21" t="n"/>
+      <c r="DL48" s="21" t="n">
+        <v>1.25</v>
+      </c>
       <c r="DM48" s="21" t="n"/>
       <c r="DN48" s="21" t="n"/>
       <c r="DO48" s="21" t="n"/>
@@ -20297,7 +20301,9 @@
       <c r="DI55" s="21" t="n"/>
       <c r="DJ55" s="21" t="n"/>
       <c r="DK55" s="21" t="n"/>
-      <c r="DL55" s="21" t="n"/>
+      <c r="DL55" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="DM55" s="21" t="n"/>
       <c r="DN55" s="21" t="n"/>
       <c r="DO55" s="21" t="n"/>
@@ -23965,7 +23971,9 @@
       <c r="DI68" s="21" t="n"/>
       <c r="DJ68" s="21" t="n"/>
       <c r="DK68" s="21" t="n"/>
-      <c r="DL68" s="21" t="n"/>
+      <c r="DL68" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="DM68" s="21" t="n">
         <v>0.5</v>
       </c>
@@ -26265,7 +26273,9 @@
       <c r="DI76" s="21" t="n"/>
       <c r="DJ76" s="21" t="n"/>
       <c r="DK76" s="21" t="n"/>
-      <c r="DL76" s="21" t="n"/>
+      <c r="DL76" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="DM76" s="21" t="n">
         <v>0.25</v>
       </c>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-06-10 22:14 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -11531,7 +11531,9 @@
       <c r="DI24" s="12" t="n"/>
       <c r="DJ24" s="12" t="n"/>
       <c r="DK24" s="12" t="n"/>
-      <c r="DL24" s="12" t="n"/>
+      <c r="DL24" s="12" t="n">
+        <v>0.25</v>
+      </c>
       <c r="DM24" s="12" t="n"/>
       <c r="DN24" s="12" t="n"/>
       <c r="DO24" s="12" t="n"/>
@@ -13994,7 +13996,7 @@
       <c r="DJ33" s="21" t="n"/>
       <c r="DK33" s="21" t="n"/>
       <c r="DL33" s="21" t="n">
-        <v>6</v>
+        <v>5.75</v>
       </c>
       <c r="DM33" s="21" t="n">
         <v>6</v>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-06-10 22:16 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -7900,7 +7900,9 @@
       <c r="DH11" s="12" t="n"/>
       <c r="DI11" s="12" t="n"/>
       <c r="DJ11" s="12" t="n"/>
-      <c r="DK11" s="12" t="n"/>
+      <c r="DK11" s="12" t="n">
+        <v>1.5</v>
+      </c>
       <c r="DL11" s="12" t="n"/>
       <c r="DM11" s="12" t="n">
         <v>0.25</v>
@@ -13994,7 +13996,9 @@
       <c r="DH33" s="21" t="n"/>
       <c r="DI33" s="21" t="n"/>
       <c r="DJ33" s="21" t="n"/>
-      <c r="DK33" s="21" t="n"/>
+      <c r="DK33" s="21" t="n">
+        <v>5.75</v>
+      </c>
       <c r="DL33" s="21" t="n">
         <v>5.75</v>
       </c>
@@ -19734,7 +19738,9 @@
       <c r="DH53" s="21" t="n"/>
       <c r="DI53" s="21" t="n"/>
       <c r="DJ53" s="21" t="n"/>
-      <c r="DK53" s="21" t="n"/>
+      <c r="DK53" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="DL53" s="21" t="n"/>
       <c r="DM53" s="21" t="n"/>
       <c r="DN53" s="21" t="n"/>
@@ -23972,7 +23978,9 @@
       <c r="DH68" s="21" t="n"/>
       <c r="DI68" s="21" t="n"/>
       <c r="DJ68" s="21" t="n"/>
-      <c r="DK68" s="21" t="n"/>
+      <c r="DK68" s="21" t="n">
+        <v>0.5</v>
+      </c>
       <c r="DL68" s="21" t="n">
         <v>0.25</v>
       </c>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-06-10 22:17 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -14003,7 +14003,7 @@
         <v>5.75</v>
       </c>
       <c r="DM33" s="21" t="n">
-        <v>6</v>
+        <v>5.5</v>
       </c>
       <c r="DN33" s="21" t="n"/>
       <c r="DO33" s="21" t="n"/>
@@ -19742,7 +19742,9 @@
         <v>0.25</v>
       </c>
       <c r="DL53" s="21" t="n"/>
-      <c r="DM53" s="21" t="n"/>
+      <c r="DM53" s="21" t="n">
+        <v>0.5</v>
+      </c>
       <c r="DN53" s="21" t="n"/>
       <c r="DO53" s="21" t="n"/>
       <c r="DP53" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-06-10 22:19 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -7896,7 +7896,9 @@
       <c r="DD11" s="12" t="n"/>
       <c r="DE11" s="19" t="n"/>
       <c r="DF11" s="12" t="n"/>
-      <c r="DG11" s="12" t="n"/>
+      <c r="DG11" s="12" t="n">
+        <v>1.75</v>
+      </c>
       <c r="DH11" s="12" t="n"/>
       <c r="DI11" s="12" t="n"/>
       <c r="DJ11" s="12" t="n"/>
@@ -13992,7 +13994,9 @@
       <c r="DD33" s="21" t="n"/>
       <c r="DE33" s="24" t="n"/>
       <c r="DF33" s="21" t="n"/>
-      <c r="DG33" s="21" t="n"/>
+      <c r="DG33" s="21" t="n">
+        <v>1.75</v>
+      </c>
       <c r="DH33" s="21" t="n"/>
       <c r="DI33" s="21" t="n"/>
       <c r="DJ33" s="21" t="n"/>
@@ -17567,7 +17571,9 @@
       <c r="DD46" s="21" t="n"/>
       <c r="DE46" s="24" t="n"/>
       <c r="DF46" s="21" t="n"/>
-      <c r="DG46" s="21" t="n"/>
+      <c r="DG46" s="21" t="n">
+        <v>1</v>
+      </c>
       <c r="DH46" s="21" t="n"/>
       <c r="DI46" s="21" t="n"/>
       <c r="DJ46" s="21" t="n"/>
@@ -19734,7 +19740,9 @@
       <c r="DD53" s="21" t="n"/>
       <c r="DE53" s="24" t="n"/>
       <c r="DF53" s="21" t="n"/>
-      <c r="DG53" s="21" t="n"/>
+      <c r="DG53" s="21" t="n">
+        <v>1.5</v>
+      </c>
       <c r="DH53" s="21" t="n"/>
       <c r="DI53" s="21" t="n"/>
       <c r="DJ53" s="21" t="n"/>
@@ -20306,7 +20314,9 @@
       <c r="DD55" s="21" t="n"/>
       <c r="DE55" s="24" t="n"/>
       <c r="DF55" s="21" t="n"/>
-      <c r="DG55" s="21" t="n"/>
+      <c r="DG55" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="DH55" s="21" t="n"/>
       <c r="DI55" s="21" t="n"/>
       <c r="DJ55" s="21" t="n"/>
@@ -23976,7 +23986,9 @@
       <c r="DD68" s="21" t="n"/>
       <c r="DE68" s="24" t="n"/>
       <c r="DF68" s="21" t="n"/>
-      <c r="DG68" s="21" t="n"/>
+      <c r="DG68" s="21" t="n">
+        <v>0.75</v>
+      </c>
       <c r="DH68" s="21" t="n"/>
       <c r="DI68" s="21" t="n"/>
       <c r="DJ68" s="21" t="n"/>
@@ -26280,7 +26292,9 @@
       <c r="DD76" s="21" t="n"/>
       <c r="DE76" s="24" t="n"/>
       <c r="DF76" s="21" t="n"/>
-      <c r="DG76" s="21" t="n"/>
+      <c r="DG76" s="21" t="n">
+        <v>1</v>
+      </c>
       <c r="DH76" s="21" t="n"/>
       <c r="DI76" s="21" t="n"/>
       <c r="DJ76" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-06-10 22:20 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -7899,7 +7899,9 @@
       <c r="DG11" s="12" t="n">
         <v>1.75</v>
       </c>
-      <c r="DH11" s="12" t="n"/>
+      <c r="DH11" s="12" t="n">
+        <v>0.25</v>
+      </c>
       <c r="DI11" s="12" t="n"/>
       <c r="DJ11" s="12" t="n"/>
       <c r="DK11" s="12" t="n">
@@ -13997,7 +13999,9 @@
       <c r="DG33" s="21" t="n">
         <v>1.75</v>
       </c>
-      <c r="DH33" s="21" t="n"/>
+      <c r="DH33" s="21" t="n">
+        <v>3</v>
+      </c>
       <c r="DI33" s="21" t="n"/>
       <c r="DJ33" s="21" t="n"/>
       <c r="DK33" s="21" t="n">
@@ -18302,7 +18306,9 @@
       <c r="DE48" s="24" t="n"/>
       <c r="DF48" s="21" t="n"/>
       <c r="DG48" s="21" t="n"/>
-      <c r="DH48" s="21" t="n"/>
+      <c r="DH48" s="21" t="n">
+        <v>3</v>
+      </c>
       <c r="DI48" s="21" t="n"/>
       <c r="DJ48" s="21" t="n"/>
       <c r="DK48" s="21" t="n"/>
@@ -19743,7 +19749,9 @@
       <c r="DG53" s="21" t="n">
         <v>1.5</v>
       </c>
-      <c r="DH53" s="21" t="n"/>
+      <c r="DH53" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="DI53" s="21" t="n"/>
       <c r="DJ53" s="21" t="n"/>
       <c r="DK53" s="21" t="n">
@@ -23989,7 +23997,9 @@
       <c r="DG68" s="21" t="n">
         <v>0.75</v>
       </c>
-      <c r="DH68" s="21" t="n"/>
+      <c r="DH68" s="21" t="n">
+        <v>0.5</v>
+      </c>
       <c r="DI68" s="21" t="n"/>
       <c r="DJ68" s="21" t="n"/>
       <c r="DK68" s="21" t="n">
@@ -26295,7 +26305,9 @@
       <c r="DG76" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="DH76" s="21" t="n"/>
+      <c r="DH76" s="21" t="n">
+        <v>1</v>
+      </c>
       <c r="DI76" s="21" t="n"/>
       <c r="DJ76" s="21" t="n"/>
       <c r="DK76" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-06-10 22:22 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -14002,7 +14002,9 @@
       <c r="DH33" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="DI33" s="21" t="n"/>
+      <c r="DI33" s="21" t="n">
+        <v>4.5</v>
+      </c>
       <c r="DJ33" s="21" t="n"/>
       <c r="DK33" s="21" t="n">
         <v>5.75</v>
@@ -19752,7 +19754,9 @@
       <c r="DH53" s="21" t="n">
         <v>0.25</v>
       </c>
-      <c r="DI53" s="21" t="n"/>
+      <c r="DI53" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="DJ53" s="21" t="n"/>
       <c r="DK53" s="21" t="n">
         <v>0.25</v>
@@ -20326,7 +20330,9 @@
         <v>0.25</v>
       </c>
       <c r="DH55" s="21" t="n"/>
-      <c r="DI55" s="21" t="n"/>
+      <c r="DI55" s="21" t="n">
+        <v>2.75</v>
+      </c>
       <c r="DJ55" s="21" t="n"/>
       <c r="DK55" s="21" t="n"/>
       <c r="DL55" s="21" t="n">
@@ -24000,7 +24006,9 @@
       <c r="DH68" s="21" t="n">
         <v>0.5</v>
       </c>
-      <c r="DI68" s="21" t="n"/>
+      <c r="DI68" s="21" t="n">
+        <v>0.5</v>
+      </c>
       <c r="DJ68" s="21" t="n"/>
       <c r="DK68" s="21" t="n">
         <v>0.5</v>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-06-10 22:23 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -7903,7 +7903,9 @@
         <v>0.25</v>
       </c>
       <c r="DI11" s="12" t="n"/>
-      <c r="DJ11" s="12" t="n"/>
+      <c r="DJ11" s="12" t="n">
+        <v>0.25</v>
+      </c>
       <c r="DK11" s="12" t="n">
         <v>1.5</v>
       </c>
@@ -14005,7 +14007,9 @@
       <c r="DI33" s="21" t="n">
         <v>4.5</v>
       </c>
-      <c r="DJ33" s="21" t="n"/>
+      <c r="DJ33" s="21" t="n">
+        <v>5.5</v>
+      </c>
       <c r="DK33" s="21" t="n">
         <v>5.75</v>
       </c>
@@ -18312,7 +18316,9 @@
         <v>3</v>
       </c>
       <c r="DI48" s="21" t="n"/>
-      <c r="DJ48" s="21" t="n"/>
+      <c r="DJ48" s="21" t="n">
+        <v>1.25</v>
+      </c>
       <c r="DK48" s="21" t="n"/>
       <c r="DL48" s="21" t="n">
         <v>1.25</v>
@@ -24009,7 +24015,9 @@
       <c r="DI68" s="21" t="n">
         <v>0.5</v>
       </c>
-      <c r="DJ68" s="21" t="n"/>
+      <c r="DJ68" s="21" t="n">
+        <v>0.75</v>
+      </c>
       <c r="DK68" s="21" t="n">
         <v>0.5</v>
       </c>
@@ -26317,7 +26325,9 @@
         <v>1</v>
       </c>
       <c r="DI76" s="21" t="n"/>
-      <c r="DJ76" s="21" t="n"/>
+      <c r="DJ76" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="DK76" s="21" t="n"/>
       <c r="DL76" s="21" t="n">
         <v>0.25</v>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-06-11 14:18 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -13708,7 +13708,9 @@
       <c r="DF32" s="21" t="n"/>
       <c r="DG32" s="21" t="n"/>
       <c r="DH32" s="21" t="n"/>
-      <c r="DI32" s="21" t="n"/>
+      <c r="DI32" s="21" t="n">
+        <v>1.5</v>
+      </c>
       <c r="DJ32" s="21" t="n"/>
       <c r="DK32" s="21" t="n"/>
       <c r="DL32" s="21" t="n"/>
@@ -14005,7 +14007,7 @@
         <v>3</v>
       </c>
       <c r="DI33" s="21" t="n">
-        <v>4.5</v>
+        <v>3</v>
       </c>
       <c r="DJ33" s="21" t="n">
         <v>5.5</v>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-06-17 20:45 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -14021,7 +14021,9 @@
       <c r="DM33" s="21" t="n">
         <v>5.5</v>
       </c>
-      <c r="DN33" s="21" t="n"/>
+      <c r="DN33" s="21" t="n">
+        <v>5.75</v>
+      </c>
       <c r="DO33" s="21" t="n"/>
       <c r="DP33" s="21" t="n"/>
       <c r="DQ33" s="21" t="n"/>
@@ -17592,7 +17594,9 @@
       <c r="DK46" s="21" t="n"/>
       <c r="DL46" s="21" t="n"/>
       <c r="DM46" s="21" t="n"/>
-      <c r="DN46" s="21" t="n"/>
+      <c r="DN46" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="DO46" s="21" t="n"/>
       <c r="DP46" s="21" t="n"/>
       <c r="DQ46" s="21" t="n"/>
@@ -18326,7 +18330,9 @@
         <v>1.25</v>
       </c>
       <c r="DM48" s="21" t="n"/>
-      <c r="DN48" s="21" t="n"/>
+      <c r="DN48" s="21" t="n">
+        <v>1.25</v>
+      </c>
       <c r="DO48" s="21" t="n"/>
       <c r="DP48" s="21" t="n"/>
       <c r="DQ48" s="21" t="n"/>
@@ -19773,7 +19779,9 @@
       <c r="DM53" s="21" t="n">
         <v>0.5</v>
       </c>
-      <c r="DN53" s="21" t="n"/>
+      <c r="DN53" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="DO53" s="21" t="n"/>
       <c r="DP53" s="21" t="n"/>
       <c r="DQ53" s="21" t="n"/>
@@ -24029,7 +24037,9 @@
       <c r="DM68" s="21" t="n">
         <v>0.5</v>
       </c>
-      <c r="DN68" s="21" t="n"/>
+      <c r="DN68" s="21" t="n">
+        <v>0.5</v>
+      </c>
       <c r="DO68" s="21" t="n"/>
       <c r="DP68" s="21" t="n"/>
       <c r="DQ68" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-06-17 20:48 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -7914,7 +7914,9 @@
         <v>0.25</v>
       </c>
       <c r="DN11" s="12" t="n"/>
-      <c r="DO11" s="12" t="n"/>
+      <c r="DO11" s="12" t="n">
+        <v>0.25</v>
+      </c>
       <c r="DP11" s="12" t="n"/>
       <c r="DQ11" s="12" t="n"/>
       <c r="DR11" s="12" t="n"/>
@@ -10174,7 +10176,9 @@
       <c r="DL19" s="12" t="n"/>
       <c r="DM19" s="12" t="n"/>
       <c r="DN19" s="12" t="n"/>
-      <c r="DO19" s="12" t="n"/>
+      <c r="DO19" s="12" t="n">
+        <v>0.75</v>
+      </c>
       <c r="DP19" s="12" t="n"/>
       <c r="DQ19" s="12" t="n"/>
       <c r="DR19" s="12" t="n"/>
@@ -14024,7 +14028,9 @@
       <c r="DN33" s="21" t="n">
         <v>5.75</v>
       </c>
-      <c r="DO33" s="21" t="n"/>
+      <c r="DO33" s="21" t="n">
+        <v>3.5</v>
+      </c>
       <c r="DP33" s="21" t="n"/>
       <c r="DQ33" s="21" t="n"/>
       <c r="DR33" s="21" t="n"/>
@@ -17597,7 +17603,9 @@
       <c r="DN46" s="21" t="n">
         <v>0.25</v>
       </c>
-      <c r="DO46" s="21" t="n"/>
+      <c r="DO46" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="DP46" s="21" t="n"/>
       <c r="DQ46" s="21" t="n"/>
       <c r="DR46" s="21" t="n"/>
@@ -18333,7 +18341,9 @@
       <c r="DN48" s="21" t="n">
         <v>1.25</v>
       </c>
-      <c r="DO48" s="21" t="n"/>
+      <c r="DO48" s="21" t="n">
+        <v>2.75</v>
+      </c>
       <c r="DP48" s="21" t="n"/>
       <c r="DQ48" s="21" t="n"/>
       <c r="DR48" s="21" t="n"/>
@@ -26348,7 +26358,9 @@
         <v>0.25</v>
       </c>
       <c r="DN76" s="21" t="n"/>
-      <c r="DO76" s="21" t="n"/>
+      <c r="DO76" s="21" t="n">
+        <v>0.5</v>
+      </c>
       <c r="DP76" s="21" t="n"/>
       <c r="DQ76" s="21" t="n"/>
       <c r="DR76" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-06-17 20:50 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -10179,7 +10179,9 @@
       <c r="DO19" s="12" t="n">
         <v>0.75</v>
       </c>
-      <c r="DP19" s="12" t="n"/>
+      <c r="DP19" s="12" t="n">
+        <v>2</v>
+      </c>
       <c r="DQ19" s="12" t="n"/>
       <c r="DR19" s="12" t="n"/>
       <c r="DS19" s="12" t="n"/>
@@ -14031,7 +14033,9 @@
       <c r="DO33" s="21" t="n">
         <v>3.5</v>
       </c>
-      <c r="DP33" s="21" t="n"/>
+      <c r="DP33" s="21" t="n">
+        <v>4.25</v>
+      </c>
       <c r="DQ33" s="21" t="n"/>
       <c r="DR33" s="21" t="n"/>
       <c r="DS33" s="21" t="n"/>
@@ -18344,7 +18348,9 @@
       <c r="DO48" s="21" t="n">
         <v>2.75</v>
       </c>
-      <c r="DP48" s="21" t="n"/>
+      <c r="DP48" s="21" t="n">
+        <v>1.25</v>
+      </c>
       <c r="DQ48" s="21" t="n"/>
       <c r="DR48" s="21" t="n"/>
       <c r="DS48" s="21" t="n"/>
@@ -24051,7 +24057,9 @@
         <v>0.5</v>
       </c>
       <c r="DO68" s="21" t="n"/>
-      <c r="DP68" s="21" t="n"/>
+      <c r="DP68" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="DQ68" s="21" t="n"/>
       <c r="DR68" s="21" t="n"/>
       <c r="DS68" s="21" t="n"/>
@@ -26361,7 +26369,9 @@
       <c r="DO76" s="21" t="n">
         <v>0.5</v>
       </c>
-      <c r="DP76" s="21" t="n"/>
+      <c r="DP76" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="DQ76" s="21" t="n"/>
       <c r="DR76" s="21" t="n"/>
       <c r="DS76" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-06-17 20:51 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -7917,7 +7917,9 @@
       <c r="DO11" s="12" t="n">
         <v>0.25</v>
       </c>
-      <c r="DP11" s="12" t="n"/>
+      <c r="DP11" s="12" t="n">
+        <v>1.5</v>
+      </c>
       <c r="DQ11" s="12" t="n"/>
       <c r="DR11" s="12" t="n"/>
       <c r="DS11" s="12" t="n"/>
@@ -14034,7 +14036,7 @@
         <v>3.5</v>
       </c>
       <c r="DP33" s="21" t="n">
-        <v>4.25</v>
+        <v>2.75</v>
       </c>
       <c r="DQ33" s="21" t="n"/>
       <c r="DR33" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-06-17 20:56 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -13726,7 +13726,9 @@
       <c r="DN32" s="21" t="n"/>
       <c r="DO32" s="21" t="n"/>
       <c r="DP32" s="21" t="n"/>
-      <c r="DQ32" s="21" t="n"/>
+      <c r="DQ32" s="21" t="n">
+        <v>1.5</v>
+      </c>
       <c r="DR32" s="21" t="n"/>
       <c r="DS32" s="21" t="n"/>
       <c r="DT32" s="21" t="n"/>
@@ -14038,7 +14040,9 @@
       <c r="DP33" s="21" t="n">
         <v>2.75</v>
       </c>
-      <c r="DQ33" s="21" t="n"/>
+      <c r="DQ33" s="21" t="n">
+        <v>2.75</v>
+      </c>
       <c r="DR33" s="21" t="n"/>
       <c r="DS33" s="21" t="n"/>
       <c r="DT33" s="21" t="n"/>
@@ -18353,7 +18357,9 @@
       <c r="DP48" s="21" t="n">
         <v>1.25</v>
       </c>
-      <c r="DQ48" s="21" t="n"/>
+      <c r="DQ48" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="DR48" s="21" t="n"/>
       <c r="DS48" s="21" t="n"/>
       <c r="DT48" s="21" t="n"/>
@@ -19802,7 +19808,9 @@
       </c>
       <c r="DO53" s="21" t="n"/>
       <c r="DP53" s="21" t="n"/>
-      <c r="DQ53" s="21" t="n"/>
+      <c r="DQ53" s="21" t="n">
+        <v>0.5</v>
+      </c>
       <c r="DR53" s="21" t="n"/>
       <c r="DS53" s="21" t="n"/>
       <c r="DT53" s="21" t="n"/>
@@ -20376,7 +20384,9 @@
       <c r="DN55" s="21" t="n"/>
       <c r="DO55" s="21" t="n"/>
       <c r="DP55" s="21" t="n"/>
-      <c r="DQ55" s="21" t="n"/>
+      <c r="DQ55" s="21" t="n">
+        <v>2</v>
+      </c>
       <c r="DR55" s="21" t="n"/>
       <c r="DS55" s="21" t="n"/>
       <c r="DT55" s="21" t="n"/>
@@ -24062,7 +24072,9 @@
       <c r="DP68" s="21" t="n">
         <v>0.25</v>
       </c>
-      <c r="DQ68" s="21" t="n"/>
+      <c r="DQ68" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="DR68" s="21" t="n"/>
       <c r="DS68" s="21" t="n"/>
       <c r="DT68" s="21" t="n"/>
@@ -26374,7 +26386,9 @@
       <c r="DP76" s="21" t="n">
         <v>0.25</v>
       </c>
-      <c r="DQ76" s="21" t="n"/>
+      <c r="DQ76" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="DR76" s="21" t="n"/>
       <c r="DS76" s="21" t="n"/>
       <c r="DT76" s="21" t="n"/>
@@ -26658,7 +26672,9 @@
       <c r="DN77" s="21" t="n"/>
       <c r="DO77" s="21" t="n"/>
       <c r="DP77" s="21" t="n"/>
-      <c r="DQ77" s="21" t="n"/>
+      <c r="DQ77" s="21" t="n">
+        <v>0.5</v>
+      </c>
       <c r="DR77" s="21" t="n"/>
       <c r="DS77" s="21" t="n"/>
       <c r="DT77" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-06-17 20:58 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -7921,7 +7921,9 @@
         <v>1.5</v>
       </c>
       <c r="DQ11" s="12" t="n"/>
-      <c r="DR11" s="12" t="n"/>
+      <c r="DR11" s="12" t="n">
+        <v>0.25</v>
+      </c>
       <c r="DS11" s="12" t="n"/>
       <c r="DT11" s="12" t="n"/>
       <c r="DU11" s="12" t="n"/>
@@ -14043,7 +14045,9 @@
       <c r="DQ33" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="DR33" s="21" t="n"/>
+      <c r="DR33" s="21" t="n">
+        <v>4</v>
+      </c>
       <c r="DS33" s="21" t="n"/>
       <c r="DT33" s="21" t="n"/>
       <c r="DU33" s="21" t="n"/>
@@ -17618,7 +17622,9 @@
       </c>
       <c r="DP46" s="21" t="n"/>
       <c r="DQ46" s="21" t="n"/>
-      <c r="DR46" s="21" t="n"/>
+      <c r="DR46" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="DS46" s="21" t="n"/>
       <c r="DT46" s="21" t="n"/>
       <c r="DU46" s="21" t="n"/>
@@ -18360,7 +18366,9 @@
       <c r="DQ48" s="21" t="n">
         <v>0.25</v>
       </c>
-      <c r="DR48" s="21" t="n"/>
+      <c r="DR48" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="DS48" s="21" t="n"/>
       <c r="DT48" s="21" t="n"/>
       <c r="DU48" s="21" t="n"/>
@@ -19811,7 +19819,9 @@
       <c r="DQ53" s="21" t="n">
         <v>0.5</v>
       </c>
-      <c r="DR53" s="21" t="n"/>
+      <c r="DR53" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="DS53" s="21" t="n"/>
       <c r="DT53" s="21" t="n"/>
       <c r="DU53" s="21" t="n"/>
@@ -20387,7 +20397,9 @@
       <c r="DQ55" s="21" t="n">
         <v>0.75</v>
       </c>
-      <c r="DR55" s="21" t="n"/>
+      <c r="DR55" s="21" t="n">
+        <v>2</v>
+      </c>
       <c r="DS55" s="21" t="n"/>
       <c r="DT55" s="21" t="n"/>
       <c r="DU55" s="21" t="n"/>
@@ -24075,7 +24087,9 @@
       <c r="DQ68" s="21" t="n">
         <v>0.25</v>
       </c>
-      <c r="DR68" s="21" t="n"/>
+      <c r="DR68" s="21" t="n">
+        <v>0.5</v>
+      </c>
       <c r="DS68" s="21" t="n"/>
       <c r="DT68" s="21" t="n"/>
       <c r="DU68" s="21" t="n"/>
@@ -26675,7 +26689,9 @@
       <c r="DQ77" s="21" t="n">
         <v>0.5</v>
       </c>
-      <c r="DR77" s="21" t="n"/>
+      <c r="DR77" s="21" t="n">
+        <v>0.5</v>
+      </c>
       <c r="DS77" s="21" t="n"/>
       <c r="DT77" s="21" t="n"/>
       <c r="DU77" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-06-17 21:00 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -14043,7 +14043,7 @@
         <v>2.75</v>
       </c>
       <c r="DQ33" s="21" t="n">
-        <v>4</v>
+        <v>4.25</v>
       </c>
       <c r="DR33" s="21" t="n">
         <v>4</v>
@@ -19817,7 +19817,7 @@
       <c r="DO53" s="21" t="n"/>
       <c r="DP53" s="21" t="n"/>
       <c r="DQ53" s="21" t="n">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="DR53" s="21" t="n">
         <v>0.25</v>
@@ -26686,9 +26686,7 @@
       <c r="DN77" s="21" t="n"/>
       <c r="DO77" s="21" t="n"/>
       <c r="DP77" s="21" t="n"/>
-      <c r="DQ77" s="21" t="n">
-        <v>0.5</v>
-      </c>
+      <c r="DQ77" s="21" t="n"/>
       <c r="DR77" s="21" t="n">
         <v>0.5</v>
       </c>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-06-30 22:03 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -7924,7 +7924,9 @@
       <c r="DR11" s="12" t="n">
         <v>0.25</v>
       </c>
-      <c r="DS11" s="12" t="n"/>
+      <c r="DS11" s="12" t="n">
+        <v>0.25</v>
+      </c>
       <c r="DT11" s="12" t="n"/>
       <c r="DU11" s="12" t="n"/>
       <c r="DV11" s="12" t="n"/>
@@ -11558,7 +11560,9 @@
       <c r="DP24" s="12" t="n"/>
       <c r="DQ24" s="12" t="n"/>
       <c r="DR24" s="12" t="n"/>
-      <c r="DS24" s="12" t="n"/>
+      <c r="DS24" s="12" t="n">
+        <v>0.25</v>
+      </c>
       <c r="DT24" s="12" t="n"/>
       <c r="DU24" s="12" t="n"/>
       <c r="DV24" s="12" t="n"/>
@@ -14048,7 +14052,9 @@
       <c r="DR33" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="DS33" s="21" t="n"/>
+      <c r="DS33" s="21" t="n">
+        <v>4.75</v>
+      </c>
       <c r="DT33" s="21" t="n"/>
       <c r="DU33" s="21" t="n"/>
       <c r="DV33" s="21" t="n"/>
@@ -17625,7 +17631,9 @@
       <c r="DR46" s="21" t="n">
         <v>0.25</v>
       </c>
-      <c r="DS46" s="21" t="n"/>
+      <c r="DS46" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="DT46" s="21" t="n"/>
       <c r="DU46" s="21" t="n"/>
       <c r="DV46" s="21" t="n"/>
@@ -18369,7 +18377,9 @@
       <c r="DR48" s="21" t="n">
         <v>0.25</v>
       </c>
-      <c r="DS48" s="21" t="n"/>
+      <c r="DS48" s="21" t="n">
+        <v>1.75</v>
+      </c>
       <c r="DT48" s="21" t="n"/>
       <c r="DU48" s="21" t="n"/>
       <c r="DV48" s="21" t="n"/>
@@ -19822,7 +19832,9 @@
       <c r="DR53" s="21" t="n">
         <v>0.25</v>
       </c>
-      <c r="DS53" s="21" t="n"/>
+      <c r="DS53" s="21" t="n">
+        <v>0.5</v>
+      </c>
       <c r="DT53" s="21" t="n"/>
       <c r="DU53" s="21" t="n"/>
       <c r="DV53" s="21" t="n"/>
@@ -20400,7 +20412,9 @@
       <c r="DR55" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="DS55" s="21" t="n"/>
+      <c r="DS55" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="DT55" s="21" t="n"/>
       <c r="DU55" s="21" t="n"/>
       <c r="DV55" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-06-30 22:05 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -14055,7 +14055,9 @@
       <c r="DS33" s="21" t="n">
         <v>4.75</v>
       </c>
-      <c r="DT33" s="21" t="n"/>
+      <c r="DT33" s="21" t="n">
+        <v>6.5</v>
+      </c>
       <c r="DU33" s="21" t="n"/>
       <c r="DV33" s="21" t="n"/>
       <c r="DW33" s="21" t="n"/>
@@ -17634,7 +17636,9 @@
       <c r="DS46" s="21" t="n">
         <v>0.25</v>
       </c>
-      <c r="DT46" s="21" t="n"/>
+      <c r="DT46" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="DU46" s="21" t="n"/>
       <c r="DV46" s="21" t="n"/>
       <c r="DW46" s="21" t="n"/>
@@ -18380,7 +18384,9 @@
       <c r="DS48" s="21" t="n">
         <v>1.75</v>
       </c>
-      <c r="DT48" s="21" t="n"/>
+      <c r="DT48" s="21" t="n">
+        <v>2.75</v>
+      </c>
       <c r="DU48" s="21" t="n"/>
       <c r="DV48" s="21" t="n"/>
       <c r="DW48" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-06-30 22:06 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -19841,7 +19841,9 @@
       <c r="DS53" s="21" t="n">
         <v>0.5</v>
       </c>
-      <c r="DT53" s="21" t="n"/>
+      <c r="DT53" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="DU53" s="21" t="n"/>
       <c r="DV53" s="21" t="n"/>
       <c r="DW53" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-06-30 22:07 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -28120,7 +28120,9 @@
       <c r="DR82" s="21" t="n"/>
       <c r="DS82" s="21" t="n"/>
       <c r="DT82" s="21" t="n"/>
-      <c r="DU82" s="21" t="n"/>
+      <c r="DU82" s="21" t="n">
+        <v>8</v>
+      </c>
       <c r="DV82" s="21" t="n"/>
       <c r="DW82" s="21" t="n"/>
       <c r="DX82" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-06-30 22:08 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -28126,7 +28126,9 @@
       <c r="DV82" s="21" t="n">
         <v>8</v>
       </c>
-      <c r="DW82" s="21" t="n"/>
+      <c r="DW82" s="21" t="n">
+        <v>8</v>
+      </c>
       <c r="DX82" s="21" t="n">
         <v>8</v>
       </c>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-06-30 22:09 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -28132,7 +28132,9 @@
       <c r="DX82" s="21" t="n">
         <v>8</v>
       </c>
-      <c r="DY82" s="21" t="n"/>
+      <c r="DY82" s="21" t="n">
+        <v>8</v>
+      </c>
       <c r="DZ82" s="21" t="n"/>
       <c r="EA82" s="24" t="n"/>
       <c r="EB82" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-06-30 22:10 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -14063,7 +14063,9 @@
       <c r="DW33" s="21" t="n"/>
       <c r="DX33" s="21" t="n"/>
       <c r="DY33" s="21" t="n"/>
-      <c r="DZ33" s="21" t="n"/>
+      <c r="DZ33" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="EA33" s="24" t="n"/>
       <c r="EB33" s="21" t="n"/>
       <c r="EC33" s="21" t="n"/>
@@ -18392,7 +18394,9 @@
       <c r="DW48" s="21" t="n"/>
       <c r="DX48" s="21" t="n"/>
       <c r="DY48" s="21" t="n"/>
-      <c r="DZ48" s="21" t="n"/>
+      <c r="DZ48" s="21" t="n">
+        <v>3.25</v>
+      </c>
       <c r="EA48" s="24" t="n"/>
       <c r="EB48" s="21" t="n"/>
       <c r="EC48" s="21" t="n"/>
@@ -19849,7 +19853,9 @@
       <c r="DW53" s="21" t="n"/>
       <c r="DX53" s="21" t="n"/>
       <c r="DY53" s="21" t="n"/>
-      <c r="DZ53" s="21" t="n"/>
+      <c r="DZ53" s="21" t="n">
+        <v>0.5</v>
+      </c>
       <c r="EA53" s="24" t="n"/>
       <c r="EB53" s="21" t="n"/>
       <c r="EC53" s="21" t="n"/>
@@ -26433,7 +26439,9 @@
       <c r="DW76" s="21" t="n"/>
       <c r="DX76" s="21" t="n"/>
       <c r="DY76" s="21" t="n"/>
-      <c r="DZ76" s="21" t="n"/>
+      <c r="DZ76" s="21" t="n">
+        <v>4</v>
+      </c>
       <c r="EA76" s="24" t="n"/>
       <c r="EB76" s="21" t="n"/>
       <c r="EC76" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-06-30 22:12 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -11570,7 +11570,9 @@
       <c r="DX24" s="12" t="n"/>
       <c r="DY24" s="12" t="n"/>
       <c r="DZ24" s="12" t="n"/>
-      <c r="EA24" s="19" t="n"/>
+      <c r="EA24" s="19" t="n">
+        <v>0.25</v>
+      </c>
       <c r="EB24" s="12" t="n"/>
       <c r="EC24" s="12" t="n"/>
       <c r="ED24" s="12" t="n"/>
@@ -14066,7 +14068,9 @@
       <c r="DZ33" s="21" t="n">
         <v>0.25</v>
       </c>
-      <c r="EA33" s="24" t="n"/>
+      <c r="EA33" s="24" t="n">
+        <v>0.5</v>
+      </c>
       <c r="EB33" s="21" t="n"/>
       <c r="EC33" s="21" t="n"/>
       <c r="ED33" s="21" t="n"/>
@@ -17647,7 +17651,9 @@
       <c r="DX46" s="21" t="n"/>
       <c r="DY46" s="21" t="n"/>
       <c r="DZ46" s="21" t="n"/>
-      <c r="EA46" s="24" t="n"/>
+      <c r="EA46" s="24" t="n">
+        <v>0.25</v>
+      </c>
       <c r="EB46" s="21" t="n"/>
       <c r="EC46" s="21" t="n"/>
       <c r="ED46" s="21" t="n"/>
@@ -18397,7 +18403,9 @@
       <c r="DZ48" s="21" t="n">
         <v>3.25</v>
       </c>
-      <c r="EA48" s="24" t="n"/>
+      <c r="EA48" s="24" t="n">
+        <v>6.5</v>
+      </c>
       <c r="EB48" s="21" t="n"/>
       <c r="EC48" s="21" t="n"/>
       <c r="ED48" s="21" t="n"/>
@@ -24686,7 +24694,9 @@
       <c r="DX70" s="21" t="n"/>
       <c r="DY70" s="21" t="n"/>
       <c r="DZ70" s="21" t="n"/>
-      <c r="EA70" s="24" t="n"/>
+      <c r="EA70" s="24" t="n">
+        <v>0.25</v>
+      </c>
       <c r="EB70" s="21" t="n"/>
       <c r="EC70" s="21" t="n"/>
       <c r="ED70" s="21" t="n"/>
@@ -26442,7 +26452,9 @@
       <c r="DZ76" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="EA76" s="24" t="n"/>
+      <c r="EA76" s="24" t="n">
+        <v>0.25</v>
+      </c>
       <c r="EB76" s="21" t="n"/>
       <c r="EC76" s="21" t="n"/>
       <c r="ED76" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-07-02 22:25 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -7936,7 +7936,9 @@
       <c r="DZ11" s="12" t="n"/>
       <c r="EA11" s="19" t="n"/>
       <c r="EB11" s="12" t="n"/>
-      <c r="EC11" s="12" t="n"/>
+      <c r="EC11" s="12" t="n">
+        <v>1.25</v>
+      </c>
       <c r="ED11" s="12" t="n"/>
       <c r="EE11" s="12" t="n"/>
       <c r="EF11" s="12" t="n"/>
@@ -11574,7 +11576,9 @@
         <v>0.25</v>
       </c>
       <c r="EB24" s="12" t="n"/>
-      <c r="EC24" s="12" t="n"/>
+      <c r="EC24" s="12" t="n">
+        <v>0.25</v>
+      </c>
       <c r="ED24" s="12" t="n"/>
       <c r="EE24" s="12" t="n"/>
       <c r="EF24" s="12" t="n"/>
@@ -14072,7 +14076,9 @@
         <v>0.5</v>
       </c>
       <c r="EB33" s="21" t="n"/>
-      <c r="EC33" s="21" t="n"/>
+      <c r="EC33" s="21" t="n">
+        <v>2.5</v>
+      </c>
       <c r="ED33" s="21" t="n"/>
       <c r="EE33" s="21" t="n"/>
       <c r="EF33" s="21" t="n"/>
@@ -27572,7 +27578,9 @@
       <c r="DZ80" s="21" t="n"/>
       <c r="EA80" s="24" t="n"/>
       <c r="EB80" s="21" t="n"/>
-      <c r="EC80" s="21" t="n"/>
+      <c r="EC80" s="21" t="n">
+        <v>4</v>
+      </c>
       <c r="ED80" s="21" t="n"/>
       <c r="EE80" s="21" t="n"/>
       <c r="EF80" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-07-07 22:09 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -27859,7 +27859,9 @@
       <c r="EA81" s="24" t="n"/>
       <c r="EB81" s="21" t="n"/>
       <c r="EC81" s="21" t="n"/>
-      <c r="ED81" s="21" t="n"/>
+      <c r="ED81" s="21" t="n">
+        <v>8</v>
+      </c>
       <c r="EE81" s="21" t="n"/>
       <c r="EF81" s="21" t="n"/>
       <c r="EG81" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-07-07 22:13 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -14075,7 +14075,9 @@
       <c r="EA33" s="24" t="n">
         <v>0.5</v>
       </c>
-      <c r="EB33" s="21" t="n"/>
+      <c r="EB33" s="21" t="n">
+        <v>2.75</v>
+      </c>
       <c r="EC33" s="21" t="n">
         <v>2.5</v>
       </c>
@@ -17660,7 +17662,9 @@
       <c r="EA46" s="24" t="n">
         <v>0.25</v>
       </c>
-      <c r="EB46" s="21" t="n"/>
+      <c r="EB46" s="21" t="n">
+        <v>0.5</v>
+      </c>
       <c r="EC46" s="21" t="n"/>
       <c r="ED46" s="21" t="n"/>
       <c r="EE46" s="21" t="n"/>
@@ -18412,7 +18416,9 @@
       <c r="EA48" s="24" t="n">
         <v>6.5</v>
       </c>
-      <c r="EB48" s="21" t="n"/>
+      <c r="EB48" s="21" t="n">
+        <v>3.5</v>
+      </c>
       <c r="EC48" s="21" t="n"/>
       <c r="ED48" s="21" t="n"/>
       <c r="EE48" s="21" t="n"/>
@@ -19871,7 +19877,9 @@
         <v>0.5</v>
       </c>
       <c r="EA53" s="24" t="n"/>
-      <c r="EB53" s="21" t="n"/>
+      <c r="EB53" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="EC53" s="21" t="n"/>
       <c r="ED53" s="21" t="n"/>
       <c r="EE53" s="21" t="n"/>
@@ -24141,7 +24149,9 @@
       <c r="DY68" s="21" t="n"/>
       <c r="DZ68" s="21" t="n"/>
       <c r="EA68" s="24" t="n"/>
-      <c r="EB68" s="21" t="n"/>
+      <c r="EB68" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="EC68" s="21" t="n"/>
       <c r="ED68" s="21" t="n"/>
       <c r="EE68" s="21" t="n"/>
@@ -26461,7 +26471,9 @@
       <c r="EA76" s="24" t="n">
         <v>0.25</v>
       </c>
-      <c r="EB76" s="21" t="n"/>
+      <c r="EB76" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="EC76" s="21" t="n"/>
       <c r="ED76" s="21" t="n"/>
       <c r="EE76" s="21" t="n"/>
@@ -27577,7 +27589,9 @@
       <c r="DY80" s="21" t="n"/>
       <c r="DZ80" s="21" t="n"/>
       <c r="EA80" s="24" t="n"/>
-      <c r="EB80" s="21" t="n"/>
+      <c r="EB80" s="21" t="n">
+        <v>0.5</v>
+      </c>
       <c r="EC80" s="21" t="n">
         <v>4</v>
       </c>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-07-07 22:19 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -14082,7 +14082,9 @@
         <v>2.5</v>
       </c>
       <c r="ED33" s="21" t="n"/>
-      <c r="EE33" s="21" t="n"/>
+      <c r="EE33" s="21" t="n">
+        <v>2.75</v>
+      </c>
       <c r="EF33" s="21" t="n"/>
       <c r="EG33" s="21" t="n"/>
       <c r="EH33" s="21" t="n"/>
@@ -18421,7 +18423,9 @@
       </c>
       <c r="EC48" s="21" t="n"/>
       <c r="ED48" s="21" t="n"/>
-      <c r="EE48" s="21" t="n"/>
+      <c r="EE48" s="21" t="n">
+        <v>1.75</v>
+      </c>
       <c r="EF48" s="21" t="n"/>
       <c r="EG48" s="21" t="n"/>
       <c r="EH48" s="21" t="n"/>
@@ -19882,7 +19886,9 @@
       </c>
       <c r="EC53" s="21" t="n"/>
       <c r="ED53" s="21" t="n"/>
-      <c r="EE53" s="21" t="n"/>
+      <c r="EE53" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="EF53" s="21" t="n"/>
       <c r="EG53" s="21" t="n"/>
       <c r="EH53" s="21" t="n"/>
@@ -27596,7 +27602,9 @@
         <v>4</v>
       </c>
       <c r="ED80" s="21" t="n"/>
-      <c r="EE80" s="21" t="n"/>
+      <c r="EE80" s="21" t="n">
+        <v>0.75</v>
+      </c>
       <c r="EF80" s="21" t="n"/>
       <c r="EG80" s="21" t="n"/>
       <c r="EH80" s="21" t="n"/>
@@ -28741,7 +28749,9 @@
       <c r="EB84" s="21" t="n"/>
       <c r="EC84" s="21" t="n"/>
       <c r="ED84" s="21" t="n"/>
-      <c r="EE84" s="21" t="n"/>
+      <c r="EE84" s="21" t="n">
+        <v>2.5</v>
+      </c>
       <c r="EF84" s="21" t="n"/>
       <c r="EG84" s="21" t="n"/>
       <c r="EH84" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-07-07 22:22 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -14085,7 +14085,9 @@
       <c r="EE33" s="21" t="n">
         <v>2.75</v>
       </c>
-      <c r="EF33" s="21" t="n"/>
+      <c r="EF33" s="21" t="n">
+        <v>3</v>
+      </c>
       <c r="EG33" s="21" t="n"/>
       <c r="EH33" s="21" t="n"/>
       <c r="EI33" s="21" t="n"/>
@@ -17670,7 +17672,9 @@
       <c r="EC46" s="21" t="n"/>
       <c r="ED46" s="21" t="n"/>
       <c r="EE46" s="21" t="n"/>
-      <c r="EF46" s="21" t="n"/>
+      <c r="EF46" s="21" t="n">
+        <v>0.5</v>
+      </c>
       <c r="EG46" s="21" t="n"/>
       <c r="EH46" s="21" t="n"/>
       <c r="EI46" s="21" t="n"/>
@@ -18426,7 +18430,9 @@
       <c r="EE48" s="21" t="n">
         <v>1.75</v>
       </c>
-      <c r="EF48" s="21" t="n"/>
+      <c r="EF48" s="21" t="n">
+        <v>3</v>
+      </c>
       <c r="EG48" s="21" t="n"/>
       <c r="EH48" s="21" t="n"/>
       <c r="EI48" s="21" t="n"/>
@@ -19889,7 +19895,9 @@
       <c r="EE53" s="21" t="n">
         <v>0.25</v>
       </c>
-      <c r="EF53" s="21" t="n"/>
+      <c r="EF53" s="21" t="n">
+        <v>0.5</v>
+      </c>
       <c r="EG53" s="21" t="n"/>
       <c r="EH53" s="21" t="n"/>
       <c r="EI53" s="21" t="n"/>
@@ -26483,7 +26491,9 @@
       <c r="EC76" s="21" t="n"/>
       <c r="ED76" s="21" t="n"/>
       <c r="EE76" s="21" t="n"/>
-      <c r="EF76" s="21" t="n"/>
+      <c r="EF76" s="21" t="n">
+        <v>0.75</v>
+      </c>
       <c r="EG76" s="21" t="n"/>
       <c r="EH76" s="21" t="n"/>
       <c r="EI76" s="21" t="n"/>
@@ -27605,7 +27615,9 @@
       <c r="EE80" s="21" t="n">
         <v>0.75</v>
       </c>
-      <c r="EF80" s="21" t="n"/>
+      <c r="EF80" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="EG80" s="21" t="n"/>
       <c r="EH80" s="21" t="n"/>
       <c r="EI80" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-07-08 14:42 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -11580,7 +11580,9 @@
         <v>0.25</v>
       </c>
       <c r="ED24" s="12" t="n"/>
-      <c r="EE24" s="12" t="n"/>
+      <c r="EE24" s="12" t="n">
+        <v>1.25</v>
+      </c>
       <c r="EF24" s="12" t="n"/>
       <c r="EG24" s="12" t="n"/>
       <c r="EH24" s="12" t="n"/>
@@ -14083,7 +14085,7 @@
       </c>
       <c r="ED33" s="21" t="n"/>
       <c r="EE33" s="21" t="n">
-        <v>2.75</v>
+        <v>1.5</v>
       </c>
       <c r="EF33" s="21" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-07-08 14:46 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -7940,7 +7940,9 @@
         <v>1.25</v>
       </c>
       <c r="ED11" s="12" t="n"/>
-      <c r="EE11" s="12" t="n"/>
+      <c r="EE11" s="12" t="n">
+        <v>1</v>
+      </c>
       <c r="EF11" s="12" t="n"/>
       <c r="EG11" s="12" t="n"/>
       <c r="EH11" s="12" t="n"/>
@@ -11581,7 +11583,7 @@
       </c>
       <c r="ED24" s="12" t="n"/>
       <c r="EE24" s="12" t="n">
-        <v>1.25</v>
+        <v>0.25</v>
       </c>
       <c r="EF24" s="12" t="n"/>
       <c r="EG24" s="12" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-07-10 23:07 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -7946,7 +7946,9 @@
       <c r="EF11" s="12" t="n"/>
       <c r="EG11" s="12" t="n"/>
       <c r="EH11" s="12" t="n"/>
-      <c r="EI11" s="12" t="n"/>
+      <c r="EI11" s="12" t="n">
+        <v>0.5</v>
+      </c>
       <c r="EJ11" s="12" t="n"/>
       <c r="EK11" s="12" t="n"/>
       <c r="EL11" s="12" t="n"/>
@@ -14094,7 +14096,9 @@
       </c>
       <c r="EG33" s="21" t="n"/>
       <c r="EH33" s="21" t="n"/>
-      <c r="EI33" s="21" t="n"/>
+      <c r="EI33" s="21" t="n">
+        <v>4</v>
+      </c>
       <c r="EJ33" s="21" t="n"/>
       <c r="EK33" s="21" t="n"/>
       <c r="EL33" s="21" t="n"/>
@@ -18439,7 +18443,9 @@
       </c>
       <c r="EG48" s="21" t="n"/>
       <c r="EH48" s="21" t="n"/>
-      <c r="EI48" s="21" t="n"/>
+      <c r="EI48" s="21" t="n">
+        <v>3.5</v>
+      </c>
       <c r="EJ48" s="21" t="n"/>
       <c r="EK48" s="21" t="n"/>
       <c r="EL48" s="21" t="n"/>
@@ -19904,7 +19910,9 @@
       </c>
       <c r="EG53" s="21" t="n"/>
       <c r="EH53" s="21" t="n"/>
-      <c r="EI53" s="21" t="n"/>
+      <c r="EI53" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="EJ53" s="21" t="n"/>
       <c r="EK53" s="21" t="n"/>
       <c r="EL53" s="21" t="n"/>
@@ -26500,7 +26508,9 @@
       </c>
       <c r="EG76" s="21" t="n"/>
       <c r="EH76" s="21" t="n"/>
-      <c r="EI76" s="21" t="n"/>
+      <c r="EI76" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="EJ76" s="21" t="n"/>
       <c r="EK76" s="21" t="n"/>
       <c r="EL76" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-07-10 23:10 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -7944,7 +7944,9 @@
         <v>1</v>
       </c>
       <c r="EF11" s="12" t="n"/>
-      <c r="EG11" s="12" t="n"/>
+      <c r="EG11" s="12" t="n">
+        <v>0.25</v>
+      </c>
       <c r="EH11" s="12" t="n"/>
       <c r="EI11" s="12" t="n">
         <v>0.5</v>
@@ -11588,7 +11590,9 @@
         <v>0.25</v>
       </c>
       <c r="EF24" s="12" t="n"/>
-      <c r="EG24" s="12" t="n"/>
+      <c r="EG24" s="12" t="n">
+        <v>0.25</v>
+      </c>
       <c r="EH24" s="12" t="n"/>
       <c r="EI24" s="12" t="n"/>
       <c r="EJ24" s="12" t="n"/>
@@ -14094,7 +14098,9 @@
       <c r="EF33" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="EG33" s="21" t="n"/>
+      <c r="EG33" s="21" t="n">
+        <v>7</v>
+      </c>
       <c r="EH33" s="21" t="n"/>
       <c r="EI33" s="21" t="n">
         <v>4</v>
@@ -26506,7 +26512,9 @@
       <c r="EF76" s="21" t="n">
         <v>0.75</v>
       </c>
-      <c r="EG76" s="21" t="n"/>
+      <c r="EG76" s="21" t="n">
+        <v>0.5</v>
+      </c>
       <c r="EH76" s="21" t="n"/>
       <c r="EI76" s="21" t="n">
         <v>0.25</v>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-07-10 23:12 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -7947,7 +7947,9 @@
       <c r="EG11" s="12" t="n">
         <v>0.25</v>
       </c>
-      <c r="EH11" s="12" t="n"/>
+      <c r="EH11" s="12" t="n">
+        <v>0.25</v>
+      </c>
       <c r="EI11" s="12" t="n">
         <v>0.5</v>
       </c>
@@ -14101,7 +14103,9 @@
       <c r="EG33" s="21" t="n">
         <v>7</v>
       </c>
-      <c r="EH33" s="21" t="n"/>
+      <c r="EH33" s="21" t="n">
+        <v>6.75</v>
+      </c>
       <c r="EI33" s="21" t="n">
         <v>4</v>
       </c>
@@ -18448,7 +18452,9 @@
         <v>3</v>
       </c>
       <c r="EG48" s="21" t="n"/>
-      <c r="EH48" s="21" t="n"/>
+      <c r="EH48" s="21" t="n">
+        <v>0.5</v>
+      </c>
       <c r="EI48" s="21" t="n">
         <v>3.5</v>
       </c>
@@ -19915,7 +19921,9 @@
         <v>0.5</v>
       </c>
       <c r="EG53" s="21" t="n"/>
-      <c r="EH53" s="21" t="n"/>
+      <c r="EH53" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="EI53" s="21" t="n">
         <v>0.25</v>
       </c>
@@ -26515,7 +26523,9 @@
       <c r="EG76" s="21" t="n">
         <v>0.5</v>
       </c>
-      <c r="EH76" s="21" t="n"/>
+      <c r="EH76" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="EI76" s="21" t="n">
         <v>0.25</v>
       </c>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-07-17 23:10 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -7953,7 +7953,9 @@
       <c r="EI11" s="12" t="n">
         <v>0.5</v>
       </c>
-      <c r="EJ11" s="12" t="n"/>
+      <c r="EJ11" s="12" t="n">
+        <v>1.5</v>
+      </c>
       <c r="EK11" s="12" t="n"/>
       <c r="EL11" s="12" t="n"/>
       <c r="EM11" s="12" t="n"/>
@@ -14109,7 +14111,9 @@
       <c r="EI33" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="EJ33" s="21" t="n"/>
+      <c r="EJ33" s="21" t="n">
+        <v>4.5</v>
+      </c>
       <c r="EK33" s="21" t="n"/>
       <c r="EL33" s="21" t="n"/>
       <c r="EM33" s="21" t="n"/>
@@ -17696,7 +17700,9 @@
       <c r="EG46" s="21" t="n"/>
       <c r="EH46" s="21" t="n"/>
       <c r="EI46" s="21" t="n"/>
-      <c r="EJ46" s="21" t="n"/>
+      <c r="EJ46" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="EK46" s="21" t="n"/>
       <c r="EL46" s="21" t="n"/>
       <c r="EM46" s="21" t="n"/>
@@ -18458,7 +18464,9 @@
       <c r="EI48" s="21" t="n">
         <v>3.5</v>
       </c>
-      <c r="EJ48" s="21" t="n"/>
+      <c r="EJ48" s="21" t="n">
+        <v>1.5</v>
+      </c>
       <c r="EK48" s="21" t="n"/>
       <c r="EL48" s="21" t="n"/>
       <c r="EM48" s="21" t="n"/>
@@ -19927,7 +19935,9 @@
       <c r="EI53" s="21" t="n">
         <v>0.25</v>
       </c>
-      <c r="EJ53" s="21" t="n"/>
+      <c r="EJ53" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="EK53" s="21" t="n"/>
       <c r="EL53" s="21" t="n"/>
       <c r="EM53" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-07-17 23:16 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -14114,7 +14114,9 @@
       <c r="EJ33" s="21" t="n">
         <v>4.5</v>
       </c>
-      <c r="EK33" s="21" t="n"/>
+      <c r="EK33" s="21" t="n">
+        <v>7</v>
+      </c>
       <c r="EL33" s="21" t="n"/>
       <c r="EM33" s="21" t="n"/>
       <c r="EN33" s="21" t="n"/>
@@ -17703,7 +17705,9 @@
       <c r="EJ46" s="21" t="n">
         <v>0.25</v>
       </c>
-      <c r="EK46" s="21" t="n"/>
+      <c r="EK46" s="21" t="n">
+        <v>1</v>
+      </c>
       <c r="EL46" s="21" t="n"/>
       <c r="EM46" s="21" t="n"/>
       <c r="EN46" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-07-17 23:17 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -10493,7 +10493,9 @@
       <c r="EI20" s="12" t="n"/>
       <c r="EJ20" s="12" t="n"/>
       <c r="EK20" s="12" t="n"/>
-      <c r="EL20" s="12" t="n"/>
+      <c r="EL20" s="12" t="n">
+        <v>2</v>
+      </c>
       <c r="EM20" s="12" t="n"/>
       <c r="EN20" s="12" t="n"/>
       <c r="EO20" s="12" t="n"/>
@@ -14117,7 +14119,9 @@
       <c r="EK33" s="21" t="n">
         <v>7</v>
       </c>
-      <c r="EL33" s="21" t="n"/>
+      <c r="EL33" s="21" t="n">
+        <v>5.5</v>
+      </c>
       <c r="EM33" s="21" t="n"/>
       <c r="EN33" s="21" t="n"/>
       <c r="EO33" s="21" t="n"/>
@@ -17708,7 +17712,9 @@
       <c r="EK46" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="EL46" s="21" t="n"/>
+      <c r="EL46" s="21" t="n">
+        <v>0.5</v>
+      </c>
       <c r="EM46" s="21" t="n"/>
       <c r="EN46" s="21" t="n"/>
       <c r="EO46" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-07-17 23:25 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -14122,7 +14122,9 @@
       <c r="EL33" s="21" t="n">
         <v>5.5</v>
       </c>
-      <c r="EM33" s="21" t="n"/>
+      <c r="EM33" s="21" t="n">
+        <v>7.25</v>
+      </c>
       <c r="EN33" s="21" t="n"/>
       <c r="EO33" s="21" t="n"/>
       <c r="EP33" s="21" t="n"/>
@@ -17715,7 +17717,9 @@
       <c r="EL46" s="21" t="n">
         <v>0.5</v>
       </c>
-      <c r="EM46" s="21" t="n"/>
+      <c r="EM46" s="21" t="n">
+        <v>0.5</v>
+      </c>
       <c r="EN46" s="21" t="n"/>
       <c r="EO46" s="21" t="n"/>
       <c r="EP46" s="21" t="n"/>
@@ -19950,7 +19954,9 @@
       </c>
       <c r="EK53" s="21" t="n"/>
       <c r="EL53" s="21" t="n"/>
-      <c r="EM53" s="21" t="n"/>
+      <c r="EM53" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="EN53" s="21" t="n"/>
       <c r="EO53" s="21" t="n"/>
       <c r="EP53" s="21" t="n"/>
@@ -24784,7 +24790,9 @@
       <c r="EJ70" s="21" t="n"/>
       <c r="EK70" s="21" t="n"/>
       <c r="EL70" s="21" t="n"/>
-      <c r="EM70" s="21" t="n"/>
+      <c r="EM70" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="EN70" s="21" t="n"/>
       <c r="EO70" s="21" t="n"/>
       <c r="EP70" s="21" t="n"/>
@@ -26552,7 +26560,9 @@
       <c r="EJ76" s="21" t="n"/>
       <c r="EK76" s="21" t="n"/>
       <c r="EL76" s="21" t="n"/>
-      <c r="EM76" s="21" t="n"/>
+      <c r="EM76" s="21" t="n">
+        <v>1.5</v>
+      </c>
       <c r="EN76" s="21" t="n"/>
       <c r="EO76" s="21" t="n"/>
       <c r="EP76" s="21" t="n"/>

</xml_diff>

<commit_message>
Update: SUrsini_2026TimeTracking.xlsx [2026-07-17 23:27 UTC]
</commit_message>
<xml_diff>
--- a/SUrsini_2026TimeTracking.xlsx
+++ b/SUrsini_2026TimeTracking.xlsx
@@ -14125,7 +14125,9 @@
       <c r="EM33" s="21" t="n">
         <v>7.25</v>
       </c>
-      <c r="EN33" s="21" t="n"/>
+      <c r="EN33" s="21" t="n">
+        <v>5.25</v>
+      </c>
       <c r="EO33" s="21" t="n"/>
       <c r="EP33" s="21" t="n"/>
       <c r="EQ33" s="21" t="n"/>
@@ -17720,7 +17722,9 @@
       <c r="EM46" s="21" t="n">
         <v>0.5</v>
       </c>
-      <c r="EN46" s="21" t="n"/>
+      <c r="EN46" s="21" t="n">
+        <v>0.5</v>
+      </c>
       <c r="EO46" s="21" t="n"/>
       <c r="EP46" s="21" t="n"/>
       <c r="EQ46" s="21" t="n"/>
@@ -18484,7 +18488,9 @@
       <c r="EK48" s="21" t="n"/>
       <c r="EL48" s="21" t="n"/>
       <c r="EM48" s="21" t="n"/>
-      <c r="EN48" s="21" t="n"/>
+      <c r="EN48" s="21" t="n">
+        <v>2</v>
+      </c>
       <c r="EO48" s="21" t="n"/>
       <c r="EP48" s="21" t="n"/>
       <c r="EQ48" s="21" t="n"/>
@@ -19957,7 +19963,9 @@
       <c r="EM53" s="21" t="n">
         <v>0.25</v>
       </c>
-      <c r="EN53" s="21" t="n"/>
+      <c r="EN53" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="EO53" s="21" t="n"/>
       <c r="EP53" s="21" t="n"/>
       <c r="EQ53" s="21" t="n"/>
@@ -24793,7 +24801,9 @@
       <c r="EM70" s="21" t="n">
         <v>0.25</v>
       </c>
-      <c r="EN70" s="21" t="n"/>
+      <c r="EN70" s="21" t="n">
+        <v>0.25</v>
+      </c>
       <c r="EO70" s="21" t="n"/>
       <c r="EP70" s="21" t="n"/>
       <c r="EQ70" s="21" t="n"/>

</xml_diff>